<commit_message>
feat: update portfolio checkpoints in spreadsheet and compiled payload
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen HUB\v3\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EDDA7D4-A05D-485A-9531-64FC0F1DA99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81CA3F6-CAAD-4972-8BAA-B84E223D9BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Custos gerais" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="359">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -814,9 +814,6 @@
     <t>welcome_video_01</t>
   </si>
   <si>
-    <t>Conheça a visão da BPlen</t>
-  </si>
-  <si>
     <t>check_in_survey</t>
   </si>
   <si>
@@ -829,9 +826,6 @@
     <t>check_in</t>
   </si>
   <si>
-    <t>Demandas e estado atual da jornada</t>
-  </si>
-  <si>
     <t>sessao_onboarding</t>
   </si>
   <si>
@@ -844,81 +838,33 @@
     <t>onboarding</t>
   </si>
   <si>
-    <t>Agende sua sessão de onboarding individual.</t>
-  </si>
-  <si>
-    <t>perfil-profissional</t>
-  </si>
-  <si>
-    <t>Perfil Profissional</t>
-  </si>
-  <si>
     <t>form</t>
   </si>
   <si>
-    <t>perfil_profissional</t>
-  </si>
-  <si>
-    <t>Preenchimento do Perfil Profissional para estruturação do posicionamento.</t>
-  </si>
-  <si>
     <t>agendar-orientacao</t>
   </si>
   <si>
-    <t>Agendar Orientação Individual</t>
-  </si>
-  <si>
     <t>orientacao-individual-posicionamento</t>
   </si>
   <si>
-    <t>Sessão individual com orientador especialista de 1h.</t>
-  </si>
-  <si>
     <t>realizar-disc</t>
   </si>
   <si>
-    <t>Responder Questionário DISC</t>
-  </si>
-  <si>
     <t>disc</t>
   </si>
   <si>
-    <t>Formulário psicométrico oficial.</t>
-  </si>
-  <si>
     <t>agendar-devolutiva</t>
   </si>
   <si>
-    <t>Agendar Devolutiva Individual</t>
-  </si>
-  <si>
     <t>devolutiva-analise-comportamental</t>
   </si>
   <si>
-    <t>Sessão com orientador especialista de 1h.</t>
-  </si>
-  <si>
-    <t>plano-carreira-form</t>
-  </si>
-  <si>
-    <t>plano_carreira</t>
-  </si>
-  <si>
-    <t>Preenchimento do formulário do Plano de Carreira.</t>
-  </si>
-  <si>
     <t>agendar-devolutiva-plano</t>
   </si>
   <si>
-    <t>Agendar Devolutiva do Plano</t>
-  </si>
-  <si>
     <t>devolutiva-plano-carreira</t>
   </si>
   <si>
-    <t>Sessão de entrega do Plano de Carreira.</t>
-  </si>
-  <si>
     <t>gdc-form</t>
   </si>
   <si>
@@ -977,6 +923,201 @@
   </si>
   <si>
     <t>Pesquisa de encerramento e consolidação de resultados.</t>
+  </si>
+  <si>
+    <t>DISC</t>
+  </si>
+  <si>
+    <t>gestao_tempo</t>
+  </si>
+  <si>
+    <t>preferencias_aprendizado</t>
+  </si>
+  <si>
+    <t>preferencias_reconhecimento</t>
+  </si>
+  <si>
+    <t>Mapa de Gestão de Tempo</t>
+  </si>
+  <si>
+    <t>Preferências de Reconhecimento</t>
+  </si>
+  <si>
+    <t>Preferências de Aprendizado</t>
+  </si>
+  <si>
+    <t>realizar_preferencias_reconhecimento</t>
+  </si>
+  <si>
+    <t>realizar_preferencias_aprendizado</t>
+  </si>
+  <si>
+    <t>realizar_gestao_tempo</t>
+  </si>
+  <si>
+    <t>survey_plano_acordos</t>
+  </si>
+  <si>
+    <t>Avisos e Acordos</t>
+  </si>
+  <si>
+    <t>realizar_survey_plano_acordos</t>
+  </si>
+  <si>
+    <t>survey_plano_fase1</t>
+  </si>
+  <si>
+    <t>survey_plano_fase4</t>
+  </si>
+  <si>
+    <t>survey_agendamento_devolutiva</t>
+  </si>
+  <si>
+    <t>survey_plano_fase2</t>
+  </si>
+  <si>
+    <t>survey_plano_fase3</t>
+  </si>
+  <si>
+    <t>realizar_survey_plano_fase1</t>
+  </si>
+  <si>
+    <t>realizar_survey_plano_fase2</t>
+  </si>
+  <si>
+    <t>realizar_survey_plano_fase3</t>
+  </si>
+  <si>
+    <t>realizar_survey_plano_fase4</t>
+  </si>
+  <si>
+    <t>Devolutiva de Análise</t>
+  </si>
+  <si>
+    <t>6.1</t>
+  </si>
+  <si>
+    <t>6.2</t>
+  </si>
+  <si>
+    <t>Definição de Objetivos</t>
+  </si>
+  <si>
+    <t>Seleção de Recursos</t>
+  </si>
+  <si>
+    <t>Plano de Ação</t>
+  </si>
+  <si>
+    <t>Consolidação do Plano</t>
+  </si>
+  <si>
+    <t>Devolutiva do Plano</t>
+  </si>
+  <si>
+    <t>Conheça o BPlen HUB</t>
+  </si>
+  <si>
+    <t>Pre-mapa do estado atual</t>
+  </si>
+  <si>
+    <t>desmistificando_candidaturas</t>
+  </si>
+  <si>
+    <t>Desmistificando: Vagas publicadas e mercado oculto</t>
+  </si>
+  <si>
+    <t>Revisão e elaboração de CV</t>
+  </si>
+  <si>
+    <t>Elaboração de PDI</t>
+  </si>
+  <si>
+    <t>Preparação para Entrevistas e Networking</t>
+  </si>
+  <si>
+    <t>revisao_curriculo</t>
+  </si>
+  <si>
+    <t>pendente</t>
+  </si>
+  <si>
+    <t>Feedback Tecnico</t>
+  </si>
+  <si>
+    <t>pre_analise_comportamental</t>
+  </si>
+  <si>
+    <t>realizar_desmistificando_candidaturas</t>
+  </si>
+  <si>
+    <t>realizar_revisao_curriculo</t>
+  </si>
+  <si>
+    <t>realizar_pre_analise_comportamental</t>
+  </si>
+  <si>
+    <t>5.1</t>
+  </si>
+  <si>
+    <t>5.2</t>
+  </si>
+  <si>
+    <t>Boas-vindas e alinhamento de expectativas</t>
+  </si>
+  <si>
+    <t>A realidade do mercado de trabalho</t>
+  </si>
+  <si>
+    <t>Revisão do perfil profissional</t>
+  </si>
+  <si>
+    <t>Elaboração do Plano de Desenvolvimento Individual</t>
+  </si>
+  <si>
+    <t>Preparação de apresentação e pitch em entrevistas</t>
+  </si>
+  <si>
+    <t>Análise Comportamental Básica</t>
+  </si>
+  <si>
+    <t>Sessão individual de feedback do PDI e perfil profissional</t>
+  </si>
+  <si>
+    <t>Avaliação de Perfil Comportamental</t>
+  </si>
+  <si>
+    <t>Mapa de preferências de reconhecimento interpessoal</t>
+  </si>
+  <si>
+    <t>Mapa de preferências de formas e habitos de aprendizado</t>
+  </si>
+  <si>
+    <t>Mapa de habitos de priorização de tarefas e tempo</t>
+  </si>
+  <si>
+    <t>Sessão individual de Devolutiva Comportamental</t>
+  </si>
+  <si>
+    <t>Avisos e cordos do processo</t>
+  </si>
+  <si>
+    <t>Definição de objetivos de carreira profissional</t>
+  </si>
+  <si>
+    <t>Seleção de recursos para utilização durante a jornada</t>
+  </si>
+  <si>
+    <t>Plano de ação para manter foco e ritmo</t>
+  </si>
+  <si>
+    <t>Consolidação do plano para ativação assertiva</t>
+  </si>
+  <si>
+    <t>Organização de materiais para sessão de devolutiva do plano</t>
+  </si>
+  <si>
+    <t>Sessão individual de devolutiva do plano</t>
   </si>
 </sst>
 </file>
@@ -1237,7 +1378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1473,11 +1614,21 @@
     <xf numFmtId="165" fontId="12" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5001,13 +5152,13 @@
     </row>
     <row r="15" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="101" t="s">
+      <c r="B16" s="103" t="s">
         <v>198</v>
       </c>
-      <c r="C16" s="102"/>
-      <c r="D16" s="102"/>
-      <c r="E16" s="102"/>
-      <c r="F16" s="102"/>
+      <c r="C16" s="104"/>
+      <c r="D16" s="104"/>
+      <c r="E16" s="104"/>
+      <c r="F16" s="104"/>
     </row>
     <row r="17" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="61" t="s">
@@ -5198,20 +5349,20 @@
       </c>
       <c r="F29" s="41"/>
     </row>
-    <row r="30" spans="2:6" s="105" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="103" t="s">
+    <row r="30" spans="2:6" s="70" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="101" t="s">
         <v>156</v>
       </c>
       <c r="C30" s="57">
         <v>3</v>
       </c>
-      <c r="D30" s="103" t="s">
+      <c r="D30" s="101" t="s">
         <v>128</v>
       </c>
-      <c r="E30" s="104" t="s">
+      <c r="E30" s="102" t="s">
         <v>128</v>
       </c>
-      <c r="F30" s="103"/>
+      <c r="F30" s="101"/>
     </row>
     <row r="31" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="25" t="s">
@@ -5229,13 +5380,13 @@
     </row>
     <row r="32" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="101" t="s">
+      <c r="B33" s="103" t="s">
         <v>216</v>
       </c>
-      <c r="C33" s="102"/>
-      <c r="D33" s="102"/>
-      <c r="E33" s="102"/>
-      <c r="F33" s="102"/>
+      <c r="C33" s="104"/>
+      <c r="D33" s="104"/>
+      <c r="E33" s="104"/>
+      <c r="F33" s="104"/>
     </row>
     <row r="34" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="61" t="s">
@@ -5503,20 +5654,20 @@
       </c>
       <c r="F50" s="41"/>
     </row>
-    <row r="51" spans="2:6" s="105" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="103" t="s">
+    <row r="51" spans="2:6" s="70" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="101" t="s">
         <v>156</v>
       </c>
       <c r="C51" s="57">
         <v>5</v>
       </c>
-      <c r="D51" s="103" t="s">
+      <c r="D51" s="101" t="s">
         <v>128</v>
       </c>
-      <c r="E51" s="104" t="s">
+      <c r="E51" s="102" t="s">
         <v>128</v>
       </c>
-      <c r="F51" s="103"/>
+      <c r="F51" s="101"/>
     </row>
     <row r="52" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="25" t="s">
@@ -5537,13 +5688,13 @@
     </row>
     <row r="54" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="101" t="s">
+      <c r="B55" s="103" t="s">
         <v>224</v>
       </c>
-      <c r="C55" s="102"/>
-      <c r="D55" s="102"/>
-      <c r="E55" s="102"/>
-      <c r="F55" s="102"/>
+      <c r="C55" s="104"/>
+      <c r="D55" s="104"/>
+      <c r="E55" s="104"/>
+      <c r="F55" s="104"/>
     </row>
     <row r="56" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="61" t="s">
@@ -5830,20 +5981,20 @@
       </c>
       <c r="F73" s="41"/>
     </row>
-    <row r="74" spans="2:6" s="105" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B74" s="103" t="s">
+    <row r="74" spans="2:6" s="70" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B74" s="101" t="s">
         <v>156</v>
       </c>
       <c r="C74" s="57">
         <v>10</v>
       </c>
-      <c r="D74" s="103" t="s">
+      <c r="D74" s="101" t="s">
         <v>128</v>
       </c>
-      <c r="E74" s="104" t="s">
+      <c r="E74" s="102" t="s">
         <v>128</v>
       </c>
-      <c r="F74" s="103"/>
+      <c r="F74" s="101"/>
     </row>
     <row r="75" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="25" t="s">
@@ -5864,13 +6015,13 @@
       </c>
     </row>
     <row r="78" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="101" t="s">
+      <c r="B78" s="103" t="s">
         <v>228</v>
       </c>
-      <c r="C78" s="102"/>
-      <c r="D78" s="102"/>
-      <c r="E78" s="102"/>
-      <c r="F78" s="102"/>
+      <c r="C78" s="104"/>
+      <c r="D78" s="104"/>
+      <c r="E78" s="104"/>
+      <c r="F78" s="104"/>
     </row>
     <row r="79" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="61" t="s">
@@ -6195,20 +6346,20 @@
       </c>
       <c r="F98" s="41"/>
     </row>
-    <row r="99" spans="2:6" s="105" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B99" s="103" t="s">
+    <row r="99" spans="2:6" s="70" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B99" s="101" t="s">
         <v>156</v>
       </c>
       <c r="C99" s="57">
         <v>12</v>
       </c>
-      <c r="D99" s="103" t="s">
+      <c r="D99" s="101" t="s">
         <v>128</v>
       </c>
-      <c r="E99" s="104" t="s">
+      <c r="E99" s="102" t="s">
         <v>128</v>
       </c>
-      <c r="F99" s="103"/>
+      <c r="F99" s="101"/>
     </row>
     <row r="100" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B100" s="25" t="s">
@@ -6224,13 +6375,13 @@
     </row>
     <row r="101" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B102" s="101" t="s">
+      <c r="B102" s="103" t="s">
         <v>232</v>
       </c>
-      <c r="C102" s="102"/>
-      <c r="D102" s="102"/>
-      <c r="E102" s="102"/>
-      <c r="F102" s="102"/>
+      <c r="C102" s="104"/>
+      <c r="D102" s="104"/>
+      <c r="E102" s="104"/>
+      <c r="F102" s="104"/>
     </row>
     <row r="103" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="61" t="s">
@@ -6573,20 +6724,20 @@
       </c>
       <c r="F123" s="41"/>
     </row>
-    <row r="124" spans="2:6" s="105" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B124" s="103" t="s">
+    <row r="124" spans="2:6" s="70" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B124" s="101" t="s">
         <v>156</v>
       </c>
       <c r="C124" s="57">
         <v>12</v>
       </c>
-      <c r="D124" s="103" t="s">
+      <c r="D124" s="101" t="s">
         <v>128</v>
       </c>
-      <c r="E124" s="104" t="s">
+      <c r="E124" s="102" t="s">
         <v>128</v>
       </c>
-      <c r="F124" s="103"/>
+      <c r="F124" s="101"/>
     </row>
     <row r="125" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B125" s="25" t="s">
@@ -7133,352 +7284,736 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="9" style="105"/>
+    <col min="5" max="5" width="32.375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>236</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>248</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>237</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>249</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>250</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>251</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>239</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A2,Jornada!A:A,0))</f>
+        <v>Onboarding</v>
+      </c>
+      <c r="C2" t="s">
         <v>253</v>
       </c>
-      <c r="C2">
+      <c r="D2" s="107">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>254</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>255</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>256</v>
       </c>
-      <c r="G2" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>239</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A3,Jornada!A:A,0))</f>
+        <v>Onboarding</v>
+      </c>
+      <c r="C3" t="s">
+        <v>257</v>
+      </c>
+      <c r="D3" s="107">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
         <v>258</v>
       </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>259</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>260</v>
       </c>
-      <c r="F3" t="s">
-        <v>261</v>
-      </c>
-      <c r="G3" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>239</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A4,Jornada!A:A,0))</f>
+        <v>Onboarding</v>
+      </c>
+      <c r="C4" t="s">
+        <v>261</v>
+      </c>
+      <c r="D4" s="107">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>262</v>
+      </c>
+      <c r="F4" t="s">
         <v>263</v>
       </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="G4" t="s">
         <v>264</v>
       </c>
-      <c r="E4" t="s">
-        <v>265</v>
-      </c>
-      <c r="F4" t="s">
-        <v>266</v>
-      </c>
-      <c r="G4" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>241</v>
       </c>
-      <c r="B5" t="s">
-        <v>268</v>
-      </c>
-      <c r="C5">
+      <c r="B5" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A5,Jornada!A:A,0))</f>
+        <v>Posicionamento de Carreira</v>
+      </c>
+      <c r="C5" s="105" t="s">
+        <v>335</v>
+      </c>
+      <c r="D5" s="108">
         <v>1</v>
       </c>
-      <c r="D5" t="s">
-        <v>269</v>
-      </c>
-      <c r="E5" t="s">
-        <v>270</v>
+      <c r="E5" s="105" t="s">
+        <v>327</v>
       </c>
       <c r="F5" t="s">
-        <v>271</v>
-      </c>
-      <c r="G5" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>259</v>
+      </c>
+      <c r="G5" s="105" t="s">
+        <v>326</v>
+      </c>
+      <c r="H5" s="105" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>241</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A6,Jornada!A:A,0))</f>
+        <v>Posicionamento de Carreira</v>
+      </c>
+      <c r="C6" s="105" t="s">
+        <v>336</v>
+      </c>
+      <c r="D6" s="108">
+        <v>2</v>
+      </c>
+      <c r="E6" s="105" t="s">
+        <v>328</v>
+      </c>
+      <c r="F6" t="s">
+        <v>259</v>
+      </c>
+      <c r="G6" s="105" t="s">
+        <v>331</v>
+      </c>
+      <c r="H6" s="105" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>241</v>
+      </c>
+      <c r="B7" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A7,Jornada!A:A,0))</f>
+        <v>Posicionamento de Carreira</v>
+      </c>
+      <c r="C7" s="105" t="s">
+        <v>332</v>
+      </c>
+      <c r="D7" s="108">
+        <v>3</v>
+      </c>
+      <c r="E7" s="105" t="s">
+        <v>329</v>
+      </c>
+      <c r="F7" t="s">
+        <v>259</v>
+      </c>
+      <c r="G7" s="105" t="s">
+        <v>332</v>
+      </c>
+      <c r="H7" s="105" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>241</v>
+      </c>
+      <c r="B8" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A8,Jornada!A:A,0))</f>
+        <v>Posicionamento de Carreira</v>
+      </c>
+      <c r="C8" s="105" t="s">
+        <v>332</v>
+      </c>
+      <c r="D8" s="108">
+        <v>4</v>
+      </c>
+      <c r="E8" s="105" t="s">
+        <v>330</v>
+      </c>
+      <c r="F8" t="s">
+        <v>259</v>
+      </c>
+      <c r="G8" s="105" t="s">
+        <v>332</v>
+      </c>
+      <c r="H8" s="105" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>241</v>
+      </c>
+      <c r="B9" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A9,Jornada!A:A,0))</f>
+        <v>Posicionamento de Carreira</v>
+      </c>
+      <c r="C9" s="105" t="s">
+        <v>337</v>
+      </c>
+      <c r="D9" s="108" t="s">
+        <v>338</v>
+      </c>
+      <c r="E9" t="s">
+        <v>333</v>
+      </c>
+      <c r="F9" t="s">
+        <v>259</v>
+      </c>
+      <c r="G9" s="105" t="s">
+        <v>334</v>
+      </c>
+      <c r="H9" s="105" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>241</v>
+      </c>
+      <c r="B10" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A10,Jornada!A:A,0))</f>
+        <v>Posicionamento de Carreira</v>
+      </c>
+      <c r="C10" t="s">
+        <v>266</v>
+      </c>
+      <c r="D10" s="107" t="s">
+        <v>339</v>
+      </c>
+      <c r="E10" t="s">
+        <v>333</v>
+      </c>
+      <c r="F10" t="s">
+        <v>259</v>
+      </c>
+      <c r="G10" t="s">
+        <v>267</v>
+      </c>
+      <c r="H10" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>242</v>
+      </c>
+      <c r="B11" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A11,Jornada!A:A,0))</f>
+        <v>Análise Comportamental</v>
+      </c>
+      <c r="C11" t="s">
+        <v>268</v>
+      </c>
+      <c r="D11" s="107">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>294</v>
+      </c>
+      <c r="F11" t="s">
+        <v>259</v>
+      </c>
+      <c r="G11" t="s">
+        <v>269</v>
+      </c>
+      <c r="H11" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>242</v>
+      </c>
+      <c r="B12" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A12,Jornada!A:A,0))</f>
+        <v>Análise Comportamental</v>
+      </c>
+      <c r="C12" s="105" t="s">
+        <v>301</v>
+      </c>
+      <c r="D12" s="108">
+        <v>2</v>
+      </c>
+      <c r="E12" s="105" t="s">
+        <v>299</v>
+      </c>
+      <c r="F12" t="s">
+        <v>259</v>
+      </c>
+      <c r="G12" s="105" t="s">
+        <v>297</v>
+      </c>
+      <c r="H12" s="105" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>242</v>
+      </c>
+      <c r="B13" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A13,Jornada!A:A,0))</f>
+        <v>Análise Comportamental</v>
+      </c>
+      <c r="C13" s="105" t="s">
+        <v>302</v>
+      </c>
+      <c r="D13" s="109">
+        <v>3</v>
+      </c>
+      <c r="E13" s="106" t="s">
+        <v>300</v>
+      </c>
+      <c r="F13" t="s">
+        <v>259</v>
+      </c>
+      <c r="G13" s="105" t="s">
+        <v>296</v>
+      </c>
+      <c r="H13" s="106" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>242</v>
+      </c>
+      <c r="B14" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A14,Jornada!A:A,0))</f>
+        <v>Análise Comportamental</v>
+      </c>
+      <c r="C14" s="105" t="s">
+        <v>303</v>
+      </c>
+      <c r="D14" s="108">
+        <v>4</v>
+      </c>
+      <c r="E14" t="s">
+        <v>298</v>
+      </c>
+      <c r="F14" t="s">
+        <v>259</v>
+      </c>
+      <c r="G14" t="s">
+        <v>295</v>
+      </c>
+      <c r="H14" s="105" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>242</v>
+      </c>
+      <c r="B15" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A15,Jornada!A:A,0))</f>
+        <v>Análise Comportamental</v>
+      </c>
+      <c r="C15" t="s">
+        <v>270</v>
+      </c>
+      <c r="D15" s="107">
+        <v>5</v>
+      </c>
+      <c r="E15" t="s">
+        <v>316</v>
+      </c>
+      <c r="F15" t="s">
+        <v>263</v>
+      </c>
+      <c r="G15" t="s">
+        <v>271</v>
+      </c>
+      <c r="H15" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>243</v>
+      </c>
+      <c r="B16" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A16,Jornada!A:A,0))</f>
+        <v>Plano de Carreira</v>
+      </c>
+      <c r="C16" t="s">
+        <v>306</v>
+      </c>
+      <c r="D16" s="107">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>305</v>
+      </c>
+      <c r="F16" t="s">
+        <v>259</v>
+      </c>
+      <c r="G16" t="s">
+        <v>304</v>
+      </c>
+      <c r="H16" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>243</v>
+      </c>
+      <c r="B17" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A17,Jornada!A:A,0))</f>
+        <v>Plano de Carreira</v>
+      </c>
+      <c r="C17" s="105" t="s">
+        <v>312</v>
+      </c>
+      <c r="D17" s="108">
+        <v>2</v>
+      </c>
+      <c r="E17" s="105" t="s">
+        <v>319</v>
+      </c>
+      <c r="F17" t="s">
+        <v>259</v>
+      </c>
+      <c r="G17" s="105" t="s">
+        <v>307</v>
+      </c>
+      <c r="H17" s="105" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>243</v>
+      </c>
+      <c r="B18" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A18,Jornada!A:A,0))</f>
+        <v>Plano de Carreira</v>
+      </c>
+      <c r="C18" s="105" t="s">
+        <v>313</v>
+      </c>
+      <c r="D18" s="108">
+        <v>3</v>
+      </c>
+      <c r="E18" s="105" t="s">
+        <v>320</v>
+      </c>
+      <c r="F18" t="s">
+        <v>259</v>
+      </c>
+      <c r="G18" s="105" t="s">
+        <v>310</v>
+      </c>
+      <c r="H18" s="105" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>243</v>
+      </c>
+      <c r="B19" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A19,Jornada!A:A,0))</f>
+        <v>Plano de Carreira</v>
+      </c>
+      <c r="C19" s="105" t="s">
+        <v>314</v>
+      </c>
+      <c r="D19" s="108">
+        <v>4</v>
+      </c>
+      <c r="E19" s="105" t="s">
+        <v>321</v>
+      </c>
+      <c r="F19" t="s">
+        <v>259</v>
+      </c>
+      <c r="G19" s="105" t="s">
+        <v>311</v>
+      </c>
+      <c r="H19" s="105" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>243</v>
+      </c>
+      <c r="B20" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A20,Jornada!A:A,0))</f>
+        <v>Plano de Carreira</v>
+      </c>
+      <c r="C20" s="105" t="s">
+        <v>315</v>
+      </c>
+      <c r="D20" s="108">
+        <v>5</v>
+      </c>
+      <c r="E20" s="105" t="s">
+        <v>322</v>
+      </c>
+      <c r="F20" t="s">
+        <v>259</v>
+      </c>
+      <c r="G20" s="105" t="s">
+        <v>308</v>
+      </c>
+      <c r="H20" s="105" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>243</v>
+      </c>
+      <c r="B21" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A21,Jornada!A:A,0))</f>
+        <v>Plano de Carreira</v>
+      </c>
+      <c r="C21" t="s">
+        <v>272</v>
+      </c>
+      <c r="D21" s="108" t="s">
+        <v>317</v>
+      </c>
+      <c r="E21" t="s">
+        <v>323</v>
+      </c>
+      <c r="F21" t="s">
+        <v>259</v>
+      </c>
+      <c r="G21" s="105" t="s">
+        <v>309</v>
+      </c>
+      <c r="H21" s="105" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>243</v>
+      </c>
+      <c r="B22" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A22,Jornada!A:A,0))</f>
+        <v>Plano de Carreira</v>
+      </c>
+      <c r="C22" t="s">
+        <v>272</v>
+      </c>
+      <c r="D22" s="107" t="s">
+        <v>318</v>
+      </c>
+      <c r="E22" t="s">
+        <v>323</v>
+      </c>
+      <c r="F22" t="s">
+        <v>263</v>
+      </c>
+      <c r="G22" t="s">
         <v>273</v>
       </c>
-      <c r="C6">
+      <c r="H22" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>244</v>
+      </c>
+      <c r="B23" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A23,Jornada!A:A,0))</f>
+        <v>Gestão e Desenvolvimento de Carreira</v>
+      </c>
+      <c r="C23" t="s">
+        <v>274</v>
+      </c>
+      <c r="D23" s="107">
+        <v>1</v>
+      </c>
+      <c r="E23" t="s">
+        <v>275</v>
+      </c>
+      <c r="F23" t="s">
+        <v>265</v>
+      </c>
+      <c r="G23" t="s">
+        <v>276</v>
+      </c>
+      <c r="H23" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>244</v>
+      </c>
+      <c r="B24" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A24,Jornada!A:A,0))</f>
+        <v>Gestão e Desenvolvimento de Carreira</v>
+      </c>
+      <c r="C24" t="s">
+        <v>278</v>
+      </c>
+      <c r="D24" s="107">
         <v>2</v>
       </c>
-      <c r="D6" t="s">
-        <v>274</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="E24" t="s">
+        <v>279</v>
+      </c>
+      <c r="F24" t="s">
+        <v>263</v>
+      </c>
+      <c r="G24" t="s">
+        <v>280</v>
+      </c>
+      <c r="H24" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>245</v>
+      </c>
+      <c r="B25" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A25,Jornada!A:A,0))</f>
+        <v>MentoCoach</v>
+      </c>
+      <c r="C25" t="s">
+        <v>282</v>
+      </c>
+      <c r="D25" s="107">
+        <v>1</v>
+      </c>
+      <c r="E25" t="s">
+        <v>283</v>
+      </c>
+      <c r="F25" t="s">
         <v>265</v>
       </c>
-      <c r="F6" t="s">
-        <v>275</v>
-      </c>
-      <c r="G6" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>242</v>
-      </c>
-      <c r="B7" t="s">
-        <v>277</v>
-      </c>
-      <c r="C7">
+      <c r="G25" t="s">
+        <v>284</v>
+      </c>
+      <c r="H25" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>245</v>
+      </c>
+      <c r="B26" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A26,Jornada!A:A,0))</f>
+        <v>MentoCoach</v>
+      </c>
+      <c r="C26" t="s">
+        <v>286</v>
+      </c>
+      <c r="D26" s="107">
+        <v>2</v>
+      </c>
+      <c r="E26" t="s">
+        <v>287</v>
+      </c>
+      <c r="F26" t="s">
+        <v>263</v>
+      </c>
+      <c r="G26" t="s">
+        <v>288</v>
+      </c>
+      <c r="H26" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>246</v>
+      </c>
+      <c r="B27" s="105" t="str">
+        <f>INDEX(Jornada!C:C,MATCH(Checkpoints!A27,Jornada!A:A,0))</f>
+        <v>Offboarding</v>
+      </c>
+      <c r="C27" t="s">
+        <v>290</v>
+      </c>
+      <c r="D27" s="107">
         <v>1</v>
       </c>
-      <c r="D7" t="s">
-        <v>278</v>
-      </c>
-      <c r="E7" t="s">
-        <v>260</v>
-      </c>
-      <c r="F7" t="s">
-        <v>279</v>
-      </c>
-      <c r="G7" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>242</v>
-      </c>
-      <c r="B8" t="s">
-        <v>281</v>
-      </c>
-      <c r="C8">
-        <v>2</v>
-      </c>
-      <c r="D8" t="s">
-        <v>282</v>
-      </c>
-      <c r="E8" t="s">
-        <v>265</v>
-      </c>
-      <c r="F8" t="s">
-        <v>283</v>
-      </c>
-      <c r="G8" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>243</v>
-      </c>
-      <c r="B9" t="s">
-        <v>285</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9" t="s">
-        <v>169</v>
-      </c>
-      <c r="E9" t="s">
-        <v>270</v>
-      </c>
-      <c r="F9" t="s">
-        <v>286</v>
-      </c>
-      <c r="G9" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>243</v>
-      </c>
-      <c r="B10" t="s">
-        <v>288</v>
-      </c>
-      <c r="C10">
-        <v>2</v>
-      </c>
-      <c r="D10" t="s">
-        <v>289</v>
-      </c>
-      <c r="E10" t="s">
-        <v>265</v>
-      </c>
-      <c r="F10" t="s">
-        <v>290</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="E27" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>244</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="F27" t="s">
+        <v>259</v>
+      </c>
+      <c r="G27" t="s">
         <v>292</v>
       </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="H27" t="s">
         <v>293</v>
-      </c>
-      <c r="E11" t="s">
-        <v>270</v>
-      </c>
-      <c r="F11" t="s">
-        <v>294</v>
-      </c>
-      <c r="G11" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>244</v>
-      </c>
-      <c r="B12" t="s">
-        <v>296</v>
-      </c>
-      <c r="C12">
-        <v>2</v>
-      </c>
-      <c r="D12" t="s">
-        <v>297</v>
-      </c>
-      <c r="E12" t="s">
-        <v>265</v>
-      </c>
-      <c r="F12" t="s">
-        <v>298</v>
-      </c>
-      <c r="G12" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>245</v>
-      </c>
-      <c r="B13" t="s">
-        <v>300</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13" t="s">
-        <v>301</v>
-      </c>
-      <c r="E13" t="s">
-        <v>270</v>
-      </c>
-      <c r="F13" t="s">
-        <v>302</v>
-      </c>
-      <c r="G13" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>245</v>
-      </c>
-      <c r="B14" t="s">
-        <v>304</v>
-      </c>
-      <c r="C14">
-        <v>2</v>
-      </c>
-      <c r="D14" t="s">
-        <v>305</v>
-      </c>
-      <c r="E14" t="s">
-        <v>265</v>
-      </c>
-      <c r="F14" t="s">
-        <v>306</v>
-      </c>
-      <c r="G14" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>246</v>
-      </c>
-      <c r="B15" t="s">
-        <v>308</v>
-      </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-      <c r="D15" t="s">
-        <v>309</v>
-      </c>
-      <c r="E15" t="s">
-        <v>260</v>
-      </c>
-      <c r="F15" t="s">
-        <v>310</v>
-      </c>
-      <c r="G15" t="s">
-        <v>311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync portfolio checkpoints and add completed CV downloads to journey
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a5263ad85f0b2806/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen HUB\v3\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{F81CA3F6-CAAD-4972-8BAA-B84E223D9BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4202CD59-E623-4657-B6F3-F3FF60DF2EBF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C5E0948-C48D-459A-A83F-4DC089C1A59F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Custos gerais" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <sheet name="Jornada" sheetId="8" r:id="rId8"/>
     <sheet name="Checkpoints" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="383">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -1045,9 +1045,6 @@
     <t>realizar_desmistificando_candidaturas</t>
   </si>
   <si>
-    <t>realizar_revisao_curriculo</t>
-  </si>
-  <si>
     <t>realizar_pre_analise_comportamental</t>
   </si>
   <si>
@@ -1163,6 +1160,36 @@
   </si>
   <si>
     <t>Central de do histórico profissional</t>
+  </si>
+  <si>
+    <t>cv_focado</t>
+  </si>
+  <si>
+    <t>3.1</t>
+  </si>
+  <si>
+    <t>3.2</t>
+  </si>
+  <si>
+    <t>3.3</t>
+  </si>
+  <si>
+    <t>perfil_profissional_publico</t>
+  </si>
+  <si>
+    <t>realizar_master_cv</t>
+  </si>
+  <si>
+    <t>realizar_cv_focado</t>
+  </si>
+  <si>
+    <t>realizar_perfil_profissional_publico</t>
+  </si>
+  <si>
+    <t>Adaptação do CV com foco no objetivo pretendido</t>
+  </si>
+  <si>
+    <t>Aplicação do CV nos perfis profissionais online</t>
   </si>
 </sst>
 </file>
@@ -1423,7 +1450,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1663,6 +1690,7 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1760,10 +1788,6 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7322,7 +7346,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9" style="70"/>
@@ -7427,7 +7451,7 @@
         <v>264</v>
       </c>
       <c r="H4" s="70" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7453,7 +7477,7 @@
         <v>326</v>
       </c>
       <c r="H5" s="70" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7464,10 +7488,10 @@
         <v>163</v>
       </c>
       <c r="C6" s="70" t="s">
+        <v>352</v>
+      </c>
+      <c r="D6" s="70" t="s">
         <v>353</v>
-      </c>
-      <c r="D6" s="70" t="s">
-        <v>354</v>
       </c>
       <c r="E6" s="70" t="s">
         <v>319</v>
@@ -7476,10 +7500,10 @@
         <v>259</v>
       </c>
       <c r="G6" s="70" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="H6" s="70" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7490,22 +7514,22 @@
         <v>163</v>
       </c>
       <c r="C7" s="70" t="s">
+        <v>355</v>
+      </c>
+      <c r="D7" s="70" t="s">
         <v>356</v>
       </c>
-      <c r="D7" s="70" t="s">
-        <v>357</v>
-      </c>
       <c r="E7" s="70" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F7" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G7" s="70" t="s">
+        <v>357</v>
+      </c>
+      <c r="H7" s="70" t="s">
         <v>358</v>
-      </c>
-      <c r="H7" s="70" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7516,22 +7540,22 @@
         <v>163</v>
       </c>
       <c r="C8" s="70" t="s">
+        <v>359</v>
+      </c>
+      <c r="D8" s="70" t="s">
         <v>360</v>
       </c>
-      <c r="D8" s="70" t="s">
-        <v>361</v>
-      </c>
       <c r="E8" s="70" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="F8" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G8" s="70" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7542,22 +7566,22 @@
         <v>163</v>
       </c>
       <c r="C9" s="70" t="s">
+        <v>362</v>
+      </c>
+      <c r="D9" s="70" t="s">
         <v>363</v>
       </c>
-      <c r="D9" s="70" t="s">
-        <v>364</v>
-      </c>
       <c r="E9" s="70" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F9" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G9" s="70" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="H9" s="70" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -7568,10 +7592,10 @@
         <v>163</v>
       </c>
       <c r="C10" s="70" t="s">
-        <v>334</v>
-      </c>
-      <c r="D10" s="70">
-        <v>3</v>
+        <v>378</v>
+      </c>
+      <c r="D10" s="70" t="s">
+        <v>374</v>
       </c>
       <c r="E10" s="70" t="s">
         <v>328</v>
@@ -7580,13 +7604,13 @@
         <v>259</v>
       </c>
       <c r="G10" s="70" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H10" s="70" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="70" t="s">
         <v>241</v>
       </c>
@@ -7594,25 +7618,25 @@
         <v>163</v>
       </c>
       <c r="C11" s="70" t="s">
-        <v>330</v>
-      </c>
-      <c r="D11" s="70">
-        <v>4</v>
+        <v>379</v>
+      </c>
+      <c r="D11" s="70" t="s">
+        <v>375</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F11" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G11" s="70" t="s">
-        <v>330</v>
+        <v>373</v>
       </c>
       <c r="H11" s="70" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="70" t="s">
         <v>241</v>
       </c>
@@ -7620,22 +7644,22 @@
         <v>163</v>
       </c>
       <c r="C12" s="70" t="s">
-        <v>335</v>
+        <v>380</v>
       </c>
       <c r="D12" s="70" t="s">
-        <v>336</v>
+        <v>376</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="F12" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G12" s="70" t="s">
-        <v>332</v>
+        <v>377</v>
       </c>
       <c r="H12" s="70" t="s">
-        <v>366</v>
+        <v>382</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -7646,77 +7670,77 @@
         <v>163</v>
       </c>
       <c r="C13" s="70" t="s">
-        <v>266</v>
-      </c>
-      <c r="D13" s="70" t="s">
-        <v>337</v>
+        <v>330</v>
+      </c>
+      <c r="D13" s="70">
+        <v>4</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="F13" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G13" s="70" t="s">
-        <v>267</v>
+        <v>330</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>367</v>
+        <v>339</v>
       </c>
     </row>
     <row r="14" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="70" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B14" s="70" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C14" s="70" t="s">
-        <v>268</v>
-      </c>
-      <c r="D14" s="70">
-        <v>1</v>
+        <v>334</v>
+      </c>
+      <c r="D14" s="70" t="s">
+        <v>335</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>294</v>
+        <v>331</v>
       </c>
       <c r="F14" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G14" s="70" t="s">
-        <v>269</v>
+        <v>332</v>
       </c>
       <c r="H14" s="70" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="70" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B15" s="70" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C15" s="70" t="s">
-        <v>301</v>
-      </c>
-      <c r="D15" s="70">
-        <v>2</v>
+        <v>266</v>
+      </c>
+      <c r="D15" s="70" t="s">
+        <v>336</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>299</v>
+        <v>331</v>
       </c>
       <c r="F15" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G15" s="70" t="s">
-        <v>297</v>
+        <v>267</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="70" t="s">
         <v>242</v>
       </c>
@@ -7724,22 +7748,22 @@
         <v>166</v>
       </c>
       <c r="C16" s="70" t="s">
-        <v>302</v>
+        <v>268</v>
       </c>
       <c r="D16" s="70">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E16" s="70" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="F16" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G16" s="70" t="s">
-        <v>296</v>
+        <v>269</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="17" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7750,25 +7774,25 @@
         <v>166</v>
       </c>
       <c r="C17" s="70" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D17" s="70">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E17" s="70" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F17" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G17" s="70" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="H17" s="70" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="70" t="s">
         <v>242</v>
       </c>
@@ -7776,74 +7800,74 @@
         <v>166</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>270</v>
+        <v>302</v>
       </c>
       <c r="D18" s="70">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E18" s="70" t="s">
-        <v>316</v>
+        <v>300</v>
       </c>
       <c r="F18" s="70" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="G18" s="70" t="s">
-        <v>271</v>
+        <v>296</v>
       </c>
       <c r="H18" s="70" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
     </row>
     <row r="19" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="70" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B19" s="70" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C19" s="70" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D19" s="70">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E19" s="70" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="F19" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G19" s="70" t="s">
-        <v>304</v>
+        <v>295</v>
       </c>
       <c r="H19" s="70" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="20" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="70" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B20" s="70" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C20" s="70" t="s">
-        <v>312</v>
+        <v>270</v>
       </c>
       <c r="D20" s="70">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E20" s="70" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="F20" s="70" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="G20" s="70" t="s">
-        <v>307</v>
+        <v>271</v>
       </c>
       <c r="H20" s="70" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7854,25 +7878,25 @@
         <v>169</v>
       </c>
       <c r="C21" s="70" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="D21" s="70">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E21" s="70" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="F21" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G21" s="70" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H21" s="70" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="70" t="s">
         <v>243</v>
       </c>
@@ -7880,25 +7904,25 @@
         <v>169</v>
       </c>
       <c r="C22" s="70" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="D22" s="70">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E22" s="70" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="F22" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G22" s="70" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="H22" s="70" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="70" t="s">
         <v>243</v>
       </c>
@@ -7906,22 +7930,22 @@
         <v>169</v>
       </c>
       <c r="C23" s="70" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D23" s="70">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E23" s="70" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F23" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G23" s="70" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H23" s="70" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -7932,22 +7956,22 @@
         <v>169</v>
       </c>
       <c r="C24" s="70" t="s">
-        <v>272</v>
-      </c>
-      <c r="D24" s="70" t="s">
-        <v>317</v>
+        <v>314</v>
+      </c>
+      <c r="D24" s="70">
+        <v>4</v>
       </c>
       <c r="E24" s="70" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="F24" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G24" s="70" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="H24" s="70" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -7958,151 +7982,203 @@
         <v>169</v>
       </c>
       <c r="C25" s="70" t="s">
-        <v>272</v>
-      </c>
-      <c r="D25" s="70" t="s">
-        <v>318</v>
+        <v>315</v>
+      </c>
+      <c r="D25" s="70">
+        <v>5</v>
       </c>
       <c r="E25" s="70" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F25" s="70" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="G25" s="70" t="s">
-        <v>273</v>
+        <v>308</v>
       </c>
       <c r="H25" s="70" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="70" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B26" s="70" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="C26" s="70" t="s">
-        <v>274</v>
-      </c>
-      <c r="D26" s="70">
-        <v>1</v>
+        <v>272</v>
+      </c>
+      <c r="D26" s="70" t="s">
+        <v>317</v>
       </c>
       <c r="E26" s="70" t="s">
-        <v>275</v>
+        <v>323</v>
       </c>
       <c r="F26" s="70" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="G26" s="70" t="s">
-        <v>276</v>
+        <v>309</v>
       </c>
       <c r="H26" s="70" t="s">
-        <v>277</v>
+        <v>350</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="70" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B27" s="70" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="C27" s="70" t="s">
-        <v>278</v>
-      </c>
-      <c r="D27" s="70">
-        <v>2</v>
+        <v>272</v>
+      </c>
+      <c r="D27" s="70" t="s">
+        <v>318</v>
       </c>
       <c r="E27" s="70" t="s">
-        <v>279</v>
+        <v>323</v>
       </c>
       <c r="F27" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G27" s="70" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="H27" s="70" t="s">
-        <v>281</v>
+        <v>351</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="70" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B28" s="70" t="s">
-        <v>113</v>
+        <v>174</v>
       </c>
       <c r="C28" s="70" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="D28" s="70">
         <v>1</v>
       </c>
       <c r="E28" s="70" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="F28" s="70" t="s">
         <v>265</v>
       </c>
       <c r="G28" s="70" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="H28" s="70" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="70" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B29" s="70" t="s">
-        <v>113</v>
+        <v>174</v>
       </c>
       <c r="C29" s="70" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="D29" s="70">
         <v>2</v>
       </c>
       <c r="E29" s="70" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="F29" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G29" s="70" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="H29" s="70" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="70" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B30" s="70" t="s">
-        <v>247</v>
+        <v>113</v>
       </c>
       <c r="C30" s="70" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="D30" s="70">
         <v>1</v>
       </c>
       <c r="E30" s="70" t="s">
+        <v>283</v>
+      </c>
+      <c r="F30" s="70" t="s">
+        <v>265</v>
+      </c>
+      <c r="G30" s="70" t="s">
+        <v>284</v>
+      </c>
+      <c r="H30" s="70" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B31" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C31" s="70" t="s">
+        <v>286</v>
+      </c>
+      <c r="D31" s="70">
+        <v>2</v>
+      </c>
+      <c r="E31" s="70" t="s">
+        <v>287</v>
+      </c>
+      <c r="F31" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G31" s="70" t="s">
+        <v>288</v>
+      </c>
+      <c r="H31" s="70" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="70" t="s">
+        <v>246</v>
+      </c>
+      <c r="B32" s="70" t="s">
+        <v>247</v>
+      </c>
+      <c r="C32" s="70" t="s">
+        <v>290</v>
+      </c>
+      <c r="D32" s="70">
+        <v>1</v>
+      </c>
+      <c r="E32" s="70" t="s">
         <v>291</v>
       </c>
-      <c r="F30" s="70" t="s">
+      <c r="F32" s="70" t="s">
         <v>259</v>
       </c>
-      <c r="G30" s="70" t="s">
+      <c r="G32" s="70" t="s">
         <v>292</v>
       </c>
-      <c r="H30" s="70" t="s">
+      <c r="H32" s="70" t="s">
         <v>293</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: sync GDC checkpoints, add calendar theme filtering, 1-to-1 shortcut, and dynamic subcheckpoints
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen HUB\v3\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C5E0948-C48D-459A-A83F-4DC089C1A59F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F32698C-664F-4EBB-8172-E004BB472FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Custos gerais" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="387">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -865,30 +865,6 @@
     <t>devolutiva-plano-carreira</t>
   </si>
   <si>
-    <t>gdc-form</t>
-  </si>
-  <si>
-    <t>Gestão de Carreira</t>
-  </si>
-  <si>
-    <t>gdc</t>
-  </si>
-  <si>
-    <t>Formulário de acompanhamento GDC.</t>
-  </si>
-  <si>
-    <t>agendar-mentorias</t>
-  </si>
-  <si>
-    <t>Agendar Mentorias</t>
-  </si>
-  <si>
-    <t>gdc-mentorias</t>
-  </si>
-  <si>
-    <t>Agendamento de sessões periódicas de mentoria.</t>
-  </si>
-  <si>
     <t>mentocoach-form</t>
   </si>
   <si>
@@ -1190,6 +1166,42 @@
   </si>
   <si>
     <t>Aplicação do CV nos perfis profissionais online</t>
+  </si>
+  <si>
+    <t>agendar-sessao</t>
+  </si>
+  <si>
+    <t>Autoconhecimento e Aprendizagem</t>
+  </si>
+  <si>
+    <t>Gestão Comportamental e Emocional</t>
+  </si>
+  <si>
+    <t>Técnicas de Posicionamento</t>
+  </si>
+  <si>
+    <t>Gestão de Tempo e Tarefas</t>
+  </si>
+  <si>
+    <t>Comunicação e Relacionamento Interpessoal</t>
+  </si>
+  <si>
+    <t>Técnicas de Negociação</t>
+  </si>
+  <si>
+    <t>Networking e Geração de Valor</t>
+  </si>
+  <si>
+    <t>Finanças para Carreira Profissional</t>
+  </si>
+  <si>
+    <t>Liderança e Autoliderança</t>
+  </si>
+  <si>
+    <t>Práticas de Melhoria Contínua</t>
+  </si>
+  <si>
+    <t>orientacao-em-grupo</t>
   </si>
 </sst>
 </file>
@@ -7346,7 +7358,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9" style="70"/>
@@ -7399,7 +7411,7 @@
         <v>256</v>
       </c>
       <c r="H2" s="70" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -7425,7 +7437,7 @@
         <v>260</v>
       </c>
       <c r="H3" s="70" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -7451,7 +7463,7 @@
         <v>264</v>
       </c>
       <c r="H4" s="70" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7462,22 +7474,22 @@
         <v>163</v>
       </c>
       <c r="C5" s="70" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="D5" s="70">
         <v>1</v>
       </c>
       <c r="E5" s="70" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="F5" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G5" s="70" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="H5" s="70" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7488,22 +7500,22 @@
         <v>163</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="D6" s="70" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="F6" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G6" s="70" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="H6" s="70" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7514,22 +7526,22 @@
         <v>163</v>
       </c>
       <c r="C7" s="70" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="D7" s="70" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="E7" s="70" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="F7" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G7" s="70" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="H7" s="70" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7540,22 +7552,22 @@
         <v>163</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="D8" s="70" t="s">
+        <v>352</v>
+      </c>
+      <c r="E8" s="70" t="s">
         <v>360</v>
-      </c>
-      <c r="E8" s="70" t="s">
-        <v>368</v>
       </c>
       <c r="F8" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G8" s="70" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7566,22 +7578,22 @@
         <v>163</v>
       </c>
       <c r="C9" s="70" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="D9" s="70" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="F9" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G9" s="70" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="H9" s="70" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -7592,25 +7604,25 @@
         <v>163</v>
       </c>
       <c r="C10" s="70" t="s">
-        <v>378</v>
+        <v>370</v>
       </c>
       <c r="D10" s="70" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="F10" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G10" s="70" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="H10" s="70" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="70" t="s">
         <v>241</v>
       </c>
@@ -7618,25 +7630,25 @@
         <v>163</v>
       </c>
       <c r="C11" s="70" t="s">
-        <v>379</v>
+        <v>371</v>
       </c>
       <c r="D11" s="70" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="F11" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G11" s="70" t="s">
+        <v>365</v>
+      </c>
+      <c r="H11" s="70" t="s">
         <v>373</v>
       </c>
-      <c r="H11" s="70" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="70" t="s">
         <v>241</v>
       </c>
@@ -7644,22 +7656,22 @@
         <v>163</v>
       </c>
       <c r="C12" s="70" t="s">
-        <v>380</v>
+        <v>372</v>
       </c>
       <c r="D12" s="70" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="F12" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G12" s="70" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="H12" s="70" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -7670,22 +7682,22 @@
         <v>163</v>
       </c>
       <c r="C13" s="70" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="D13" s="70">
         <v>4</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="F13" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G13" s="70" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
     </row>
     <row r="14" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7696,22 +7708,22 @@
         <v>163</v>
       </c>
       <c r="C14" s="70" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="D14" s="70" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="F14" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G14" s="70" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="H14" s="70" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -7725,10 +7737,10 @@
         <v>266</v>
       </c>
       <c r="D15" s="70" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="F15" s="70" t="s">
         <v>259</v>
@@ -7737,7 +7749,7 @@
         <v>267</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
     </row>
     <row r="16" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7754,7 +7766,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="70" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="F16" s="70" t="s">
         <v>259</v>
@@ -7763,7 +7775,7 @@
         <v>269</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
     </row>
     <row r="17" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7774,22 +7786,22 @@
         <v>166</v>
       </c>
       <c r="C17" s="70" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="D17" s="70">
         <v>2</v>
       </c>
       <c r="E17" s="70" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="F17" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G17" s="70" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="H17" s="70" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -7800,22 +7812,22 @@
         <v>166</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="D18" s="70">
         <v>3</v>
       </c>
       <c r="E18" s="70" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="F18" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G18" s="70" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="H18" s="70" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
     </row>
     <row r="19" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7826,22 +7838,22 @@
         <v>166</v>
       </c>
       <c r="C19" s="70" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="D19" s="70">
         <v>4</v>
       </c>
       <c r="E19" s="70" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="F19" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G19" s="70" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="H19" s="70" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
     </row>
     <row r="20" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7858,7 +7870,7 @@
         <v>5</v>
       </c>
       <c r="E20" s="70" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="F20" s="70" t="s">
         <v>263</v>
@@ -7867,7 +7879,7 @@
         <v>271</v>
       </c>
       <c r="H20" s="70" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
     </row>
     <row r="21" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7878,22 +7890,22 @@
         <v>169</v>
       </c>
       <c r="C21" s="70" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="D21" s="70">
         <v>1</v>
       </c>
       <c r="E21" s="70" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="F21" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G21" s="70" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="H21" s="70" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
     </row>
     <row r="22" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7904,22 +7916,22 @@
         <v>169</v>
       </c>
       <c r="C22" s="70" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="D22" s="70">
         <v>2</v>
       </c>
       <c r="E22" s="70" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="F22" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G22" s="70" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="H22" s="70" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
     </row>
     <row r="23" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7930,22 +7942,22 @@
         <v>169</v>
       </c>
       <c r="C23" s="70" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="D23" s="70">
         <v>3</v>
       </c>
       <c r="E23" s="70" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="F23" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G23" s="70" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="H23" s="70" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -7956,22 +7968,22 @@
         <v>169</v>
       </c>
       <c r="C24" s="70" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="D24" s="70">
         <v>4</v>
       </c>
       <c r="E24" s="70" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="F24" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G24" s="70" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="H24" s="70" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -7982,22 +7994,22 @@
         <v>169</v>
       </c>
       <c r="C25" s="70" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="D25" s="70">
         <v>5</v>
       </c>
       <c r="E25" s="70" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="F25" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G25" s="70" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="H25" s="70" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -8011,19 +8023,19 @@
         <v>272</v>
       </c>
       <c r="D26" s="70" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="E26" s="70" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="F26" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G26" s="70" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="H26" s="70" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -8037,10 +8049,10 @@
         <v>272</v>
       </c>
       <c r="D27" s="70" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="E27" s="70" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="F27" s="70" t="s">
         <v>263</v>
@@ -8049,7 +8061,7 @@
         <v>273</v>
       </c>
       <c r="H27" s="70" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -8060,23 +8072,21 @@
         <v>174</v>
       </c>
       <c r="C28" s="70" t="s">
-        <v>274</v>
+        <v>375</v>
       </c>
       <c r="D28" s="70">
         <v>1</v>
       </c>
       <c r="E28" s="70" t="s">
-        <v>275</v>
+        <v>376</v>
       </c>
       <c r="F28" s="70" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="G28" s="70" t="s">
-        <v>276</v>
-      </c>
-      <c r="H28" s="70" t="s">
-        <v>277</v>
-      </c>
+        <v>386</v>
+      </c>
+      <c r="H28" s="70"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="70" t="s">
@@ -8086,100 +8096,290 @@
         <v>174</v>
       </c>
       <c r="C29" s="70" t="s">
-        <v>278</v>
+        <v>375</v>
       </c>
       <c r="D29" s="70">
         <v>2</v>
       </c>
       <c r="E29" s="70" t="s">
-        <v>279</v>
+        <v>377</v>
       </c>
       <c r="F29" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G29" s="70" t="s">
-        <v>280</v>
-      </c>
-      <c r="H29" s="70" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+      <c r="H29" s="70"/>
+    </row>
+    <row r="30" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="70" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B30" s="70" t="s">
-        <v>113</v>
+        <v>174</v>
       </c>
       <c r="C30" s="70" t="s">
-        <v>282</v>
+        <v>375</v>
       </c>
       <c r="D30" s="70">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E30" s="70" t="s">
-        <v>283</v>
+        <v>378</v>
       </c>
       <c r="F30" s="70" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="G30" s="70" t="s">
-        <v>284</v>
-      </c>
-      <c r="H30" s="70" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+      <c r="H30" s="70"/>
+    </row>
+    <row r="31" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="70" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B31" s="70" t="s">
-        <v>113</v>
+        <v>174</v>
       </c>
       <c r="C31" s="70" t="s">
-        <v>286</v>
+        <v>375</v>
       </c>
       <c r="D31" s="70">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E31" s="70" t="s">
-        <v>287</v>
+        <v>379</v>
       </c>
       <c r="F31" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G31" s="70" t="s">
-        <v>288</v>
-      </c>
-      <c r="H31" s="70" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+      <c r="H31" s="70"/>
+    </row>
+    <row r="32" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="70" t="s">
+        <v>244</v>
+      </c>
+      <c r="B32" s="70" t="s">
+        <v>174</v>
+      </c>
+      <c r="C32" s="70" t="s">
+        <v>375</v>
+      </c>
+      <c r="D32" s="70">
+        <v>5</v>
+      </c>
+      <c r="E32" s="70" t="s">
+        <v>380</v>
+      </c>
+      <c r="F32" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G32" s="70" t="s">
+        <v>386</v>
+      </c>
+      <c r="H32" s="70"/>
+    </row>
+    <row r="33" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="70" t="s">
+        <v>244</v>
+      </c>
+      <c r="B33" s="70" t="s">
+        <v>174</v>
+      </c>
+      <c r="C33" s="70" t="s">
+        <v>375</v>
+      </c>
+      <c r="D33" s="70">
+        <v>6</v>
+      </c>
+      <c r="E33" s="70" t="s">
+        <v>381</v>
+      </c>
+      <c r="F33" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G33" s="70" t="s">
+        <v>386</v>
+      </c>
+      <c r="H33" s="70"/>
+    </row>
+    <row r="34" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="70" t="s">
+        <v>244</v>
+      </c>
+      <c r="B34" s="70" t="s">
+        <v>174</v>
+      </c>
+      <c r="C34" s="70" t="s">
+        <v>375</v>
+      </c>
+      <c r="D34" s="70">
+        <v>7</v>
+      </c>
+      <c r="E34" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="F34" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G34" s="70" t="s">
+        <v>386</v>
+      </c>
+      <c r="H34" s="70"/>
+    </row>
+    <row r="35" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="70" t="s">
+        <v>244</v>
+      </c>
+      <c r="B35" s="70" t="s">
+        <v>174</v>
+      </c>
+      <c r="C35" s="70" t="s">
+        <v>375</v>
+      </c>
+      <c r="D35" s="70">
+        <v>8</v>
+      </c>
+      <c r="E35" s="70" t="s">
+        <v>383</v>
+      </c>
+      <c r="F35" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G35" s="70" t="s">
+        <v>386</v>
+      </c>
+      <c r="H35" s="70"/>
+    </row>
+    <row r="36" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="70" t="s">
+        <v>244</v>
+      </c>
+      <c r="B36" s="70" t="s">
+        <v>174</v>
+      </c>
+      <c r="C36" s="70" t="s">
+        <v>375</v>
+      </c>
+      <c r="D36" s="70">
+        <v>9</v>
+      </c>
+      <c r="E36" s="70" t="s">
+        <v>384</v>
+      </c>
+      <c r="F36" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G36" s="70" t="s">
+        <v>386</v>
+      </c>
+      <c r="H36" s="70"/>
+    </row>
+    <row r="37" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="70" t="s">
+        <v>244</v>
+      </c>
+      <c r="B37" s="70" t="s">
+        <v>174</v>
+      </c>
+      <c r="C37" s="70" t="s">
+        <v>375</v>
+      </c>
+      <c r="D37" s="70">
+        <v>10</v>
+      </c>
+      <c r="E37" s="70" t="s">
+        <v>385</v>
+      </c>
+      <c r="F37" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G37" s="70" t="s">
+        <v>386</v>
+      </c>
+      <c r="H37" s="70"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B38" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" s="70" t="s">
+        <v>274</v>
+      </c>
+      <c r="D38" s="70">
+        <v>1</v>
+      </c>
+      <c r="E38" s="70" t="s">
+        <v>275</v>
+      </c>
+      <c r="F38" s="70" t="s">
+        <v>265</v>
+      </c>
+      <c r="G38" s="70" t="s">
+        <v>276</v>
+      </c>
+      <c r="H38" s="70" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B39" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C39" s="70" t="s">
+        <v>278</v>
+      </c>
+      <c r="D39" s="70">
+        <v>2</v>
+      </c>
+      <c r="E39" s="70" t="s">
+        <v>279</v>
+      </c>
+      <c r="F39" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G39" s="70" t="s">
+        <v>280</v>
+      </c>
+      <c r="H39" s="70" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="70" t="s">
         <v>246</v>
       </c>
-      <c r="B32" s="70" t="s">
+      <c r="B40" s="70" t="s">
         <v>247</v>
       </c>
-      <c r="C32" s="70" t="s">
-        <v>290</v>
-      </c>
-      <c r="D32" s="70">
+      <c r="C40" s="70" t="s">
+        <v>282</v>
+      </c>
+      <c r="D40" s="70">
         <v>1</v>
       </c>
-      <c r="E32" s="70" t="s">
-        <v>291</v>
-      </c>
-      <c r="F32" s="70" t="s">
+      <c r="E40" s="70" t="s">
+        <v>283</v>
+      </c>
+      <c r="F40" s="70" t="s">
         <v>259</v>
       </c>
-      <c r="G32" s="70" t="s">
-        <v>292</v>
-      </c>
-      <c r="H32" s="70" t="s">
-        <v>293</v>
+      <c r="G40" s="70" t="s">
+        <v>284</v>
+      </c>
+      <c r="H40" s="70" t="s">
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: sync updated portfolio_bplen Excel sheet and compile payloads
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen HUB\v3\portfolio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a5263ad85f0b2806/Área de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F32698C-664F-4EBB-8172-E004BB472FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{5F32698C-664F-4EBB-8172-E004BB472FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BC574CD-1666-4CD6-AC4F-A84C2C262098}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Custos gerais" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="392">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -838,15 +838,6 @@
     <t>onboarding</t>
   </si>
   <si>
-    <t>form</t>
-  </si>
-  <si>
-    <t>agendar-orientacao</t>
-  </si>
-  <si>
-    <t>orientacao-individual-posicionamento</t>
-  </si>
-  <si>
     <t>realizar-disc</t>
   </si>
   <si>
@@ -865,30 +856,6 @@
     <t>devolutiva-plano-carreira</t>
   </si>
   <si>
-    <t>mentocoach-form</t>
-  </si>
-  <si>
-    <t>Acompanhamento MentoCoach</t>
-  </si>
-  <si>
-    <t>mentocoach</t>
-  </si>
-  <si>
-    <t>Formulário de autoavaliação MentoCoach.</t>
-  </si>
-  <si>
-    <t>agendar-sessoes</t>
-  </si>
-  <si>
-    <t>Agendar Sessões de Coaching</t>
-  </si>
-  <si>
-    <t>mentocoach-sessoes</t>
-  </si>
-  <si>
-    <t>Agendamento das sessões individuais de coaching de alta performance.</t>
-  </si>
-  <si>
     <t>offboarding-survey</t>
   </si>
   <si>
@@ -898,9 +865,6 @@
     <t>offboarding_survey</t>
   </si>
   <si>
-    <t>Pesquisa de encerramento e consolidação de resultados.</t>
-  </si>
-  <si>
     <t>DISC</t>
   </si>
   <si>
@@ -1009,9 +973,6 @@
     <t>Preparação para Entrevistas e Networking</t>
   </si>
   <si>
-    <t>pendente</t>
-  </si>
-  <si>
     <t>Feedback Tecnico</t>
   </si>
   <si>
@@ -1114,12 +1075,6 @@
     <t>survey_pdi_fase4</t>
   </si>
   <si>
-    <t>Analise Comportamental Basica</t>
-  </si>
-  <si>
-    <t>Sessao individual de feedback do PDI e perfil profissional</t>
-  </si>
-  <si>
     <t>Seleção de recursos e habilidades</t>
   </si>
   <si>
@@ -1202,6 +1157,66 @@
   </si>
   <si>
     <t>orientacao-em-grupo</t>
+  </si>
+  <si>
+    <t>preparacao_entrevistas_networking</t>
+  </si>
+  <si>
+    <t>realizar_preparacao_entrevistas_networking</t>
+  </si>
+  <si>
+    <t>Sessão de feedback do Posicionamento Profissional</t>
+  </si>
+  <si>
+    <t>agendar-feedback-posicionamento-profissional</t>
+  </si>
+  <si>
+    <t>feedback-posicionamento-profissional</t>
+  </si>
+  <si>
+    <t>Análise Comportamental Básica</t>
+  </si>
+  <si>
+    <t>Avaliação de Perfil Comportamental (DISC)</t>
+  </si>
+  <si>
+    <t>sessao-mentocoach</t>
+  </si>
+  <si>
+    <t>agendar-sessao-mentocoach</t>
+  </si>
+  <si>
+    <t>Sessões de MentoCoach</t>
+  </si>
+  <si>
+    <t>MentoCoach Dashboard</t>
+  </si>
+  <si>
+    <t>dashboard</t>
+  </si>
+  <si>
+    <t>mentocoach-dashboard</t>
+  </si>
+  <si>
+    <t>realizar-mentocoach-dashboard</t>
+  </si>
+  <si>
+    <t>Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>Acompanhamento do Progresso</t>
+  </si>
+  <si>
+    <t>Sessão de Offboarding</t>
+  </si>
+  <si>
+    <t>offboarding</t>
+  </si>
+  <si>
+    <t>Encerramento e alinhamento de próximos passos</t>
+  </si>
+  <si>
+    <t>Avalição de encerramento e consolidação de resultados.</t>
   </si>
 </sst>
 </file>
@@ -7358,7 +7373,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9" style="70"/>
@@ -7411,7 +7426,7 @@
         <v>256</v>
       </c>
       <c r="H2" s="70" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -7437,7 +7452,7 @@
         <v>260</v>
       </c>
       <c r="H3" s="70" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -7463,7 +7478,7 @@
         <v>264</v>
       </c>
       <c r="H4" s="70" t="s">
-        <v>329</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7474,22 +7489,22 @@
         <v>163</v>
       </c>
       <c r="C5" s="70" t="s">
-        <v>325</v>
+        <v>312</v>
       </c>
       <c r="D5" s="70">
         <v>1</v>
       </c>
       <c r="E5" s="70" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="F5" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G5" s="70" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="H5" s="70" t="s">
-        <v>330</v>
+        <v>317</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7500,22 +7515,22 @@
         <v>163</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>344</v>
+        <v>331</v>
       </c>
       <c r="D6" s="70" t="s">
-        <v>345</v>
+        <v>332</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="F6" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G6" s="70" t="s">
-        <v>346</v>
+        <v>333</v>
       </c>
       <c r="H6" s="70" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7526,22 +7541,22 @@
         <v>163</v>
       </c>
       <c r="C7" s="70" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
       <c r="D7" s="70" t="s">
-        <v>348</v>
+        <v>335</v>
       </c>
       <c r="E7" s="70" t="s">
-        <v>359</v>
+        <v>344</v>
       </c>
       <c r="F7" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G7" s="70" t="s">
-        <v>349</v>
+        <v>336</v>
       </c>
       <c r="H7" s="70" t="s">
-        <v>350</v>
+        <v>337</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7552,22 +7567,22 @@
         <v>163</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>351</v>
+        <v>338</v>
       </c>
       <c r="D8" s="70" t="s">
-        <v>352</v>
+        <v>339</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>360</v>
+        <v>345</v>
       </c>
       <c r="F8" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G8" s="70" t="s">
-        <v>353</v>
+        <v>340</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>360</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7578,22 +7593,22 @@
         <v>163</v>
       </c>
       <c r="C9" s="70" t="s">
-        <v>354</v>
+        <v>341</v>
       </c>
       <c r="D9" s="70" t="s">
-        <v>355</v>
+        <v>342</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>361</v>
+        <v>346</v>
       </c>
       <c r="F9" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G9" s="70" t="s">
-        <v>356</v>
+        <v>343</v>
       </c>
       <c r="H9" s="70" t="s">
-        <v>363</v>
+        <v>348</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -7604,22 +7619,22 @@
         <v>163</v>
       </c>
       <c r="C10" s="70" t="s">
-        <v>370</v>
+        <v>355</v>
       </c>
       <c r="D10" s="70" t="s">
-        <v>366</v>
+        <v>351</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="F10" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G10" s="70" t="s">
-        <v>362</v>
+        <v>347</v>
       </c>
       <c r="H10" s="70" t="s">
-        <v>364</v>
+        <v>349</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7630,22 +7645,22 @@
         <v>163</v>
       </c>
       <c r="C11" s="70" t="s">
-        <v>371</v>
+        <v>356</v>
       </c>
       <c r="D11" s="70" t="s">
-        <v>367</v>
+        <v>352</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="F11" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G11" s="70" t="s">
-        <v>365</v>
+        <v>350</v>
       </c>
       <c r="H11" s="70" t="s">
-        <v>373</v>
+        <v>358</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7656,22 +7671,22 @@
         <v>163</v>
       </c>
       <c r="C12" s="70" t="s">
-        <v>372</v>
+        <v>357</v>
       </c>
       <c r="D12" s="70" t="s">
-        <v>368</v>
+        <v>353</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="F12" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G12" s="70" t="s">
-        <v>369</v>
+        <v>354</v>
       </c>
       <c r="H12" s="70" t="s">
-        <v>374</v>
+        <v>359</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -7682,22 +7697,22 @@
         <v>163</v>
       </c>
       <c r="C13" s="70" t="s">
-        <v>322</v>
+        <v>373</v>
       </c>
       <c r="D13" s="70">
         <v>4</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="F13" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G13" s="70" t="s">
-        <v>322</v>
+        <v>372</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>331</v>
+        <v>318</v>
       </c>
     </row>
     <row r="14" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7708,22 +7723,22 @@
         <v>163</v>
       </c>
       <c r="C14" s="70" t="s">
-        <v>326</v>
+        <v>313</v>
       </c>
       <c r="D14" s="70" t="s">
-        <v>327</v>
+        <v>314</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>323</v>
+        <v>310</v>
       </c>
       <c r="F14" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G14" s="70" t="s">
-        <v>324</v>
+        <v>311</v>
       </c>
       <c r="H14" s="70" t="s">
-        <v>357</v>
+        <v>377</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -7734,22 +7749,22 @@
         <v>163</v>
       </c>
       <c r="C15" s="70" t="s">
-        <v>266</v>
+        <v>375</v>
       </c>
       <c r="D15" s="70" t="s">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>323</v>
+        <v>310</v>
       </c>
       <c r="F15" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G15" s="70" t="s">
-        <v>267</v>
+        <v>376</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>358</v>
+        <v>374</v>
       </c>
     </row>
     <row r="16" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7760,22 +7775,22 @@
         <v>166</v>
       </c>
       <c r="C16" s="70" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D16" s="70">
         <v>1</v>
       </c>
       <c r="E16" s="70" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="F16" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G16" s="70" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>332</v>
+        <v>319</v>
       </c>
     </row>
     <row r="17" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7786,22 +7801,22 @@
         <v>166</v>
       </c>
       <c r="C17" s="70" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="D17" s="70">
         <v>2</v>
       </c>
       <c r="E17" s="70" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
       <c r="F17" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G17" s="70" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
       <c r="H17" s="70" t="s">
-        <v>333</v>
+        <v>320</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -7812,22 +7827,22 @@
         <v>166</v>
       </c>
       <c r="C18" s="70" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
       <c r="D18" s="70">
         <v>3</v>
       </c>
       <c r="E18" s="70" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="F18" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G18" s="70" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="H18" s="70" t="s">
-        <v>334</v>
+        <v>321</v>
       </c>
     </row>
     <row r="19" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7838,22 +7853,22 @@
         <v>166</v>
       </c>
       <c r="C19" s="70" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="D19" s="70">
         <v>4</v>
       </c>
       <c r="E19" s="70" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="F19" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G19" s="70" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="H19" s="70" t="s">
-        <v>335</v>
+        <v>322</v>
       </c>
     </row>
     <row r="20" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7864,22 +7879,22 @@
         <v>166</v>
       </c>
       <c r="C20" s="70" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D20" s="70">
         <v>5</v>
       </c>
       <c r="E20" s="70" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="F20" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G20" s="70" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="H20" s="70" t="s">
-        <v>336</v>
+        <v>323</v>
       </c>
     </row>
     <row r="21" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7890,22 +7905,22 @@
         <v>169</v>
       </c>
       <c r="C21" s="70" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="D21" s="70">
         <v>1</v>
       </c>
       <c r="E21" s="70" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="F21" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G21" s="70" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="H21" s="70" t="s">
-        <v>337</v>
+        <v>324</v>
       </c>
     </row>
     <row r="22" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7916,22 +7931,22 @@
         <v>169</v>
       </c>
       <c r="C22" s="70" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="D22" s="70">
         <v>2</v>
       </c>
       <c r="E22" s="70" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="F22" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G22" s="70" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="H22" s="70" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
     </row>
     <row r="23" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7942,22 +7957,22 @@
         <v>169</v>
       </c>
       <c r="C23" s="70" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="D23" s="70">
         <v>3</v>
       </c>
       <c r="E23" s="70" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="F23" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G23" s="70" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="H23" s="70" t="s">
-        <v>339</v>
+        <v>326</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -7968,22 +7983,22 @@
         <v>169</v>
       </c>
       <c r="C24" s="70" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="D24" s="70">
         <v>4</v>
       </c>
       <c r="E24" s="70" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="F24" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G24" s="70" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="H24" s="70" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -7994,22 +8009,22 @@
         <v>169</v>
       </c>
       <c r="C25" s="70" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="D25" s="70">
         <v>5</v>
       </c>
       <c r="E25" s="70" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="F25" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G25" s="70" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
       <c r="H25" s="70" t="s">
-        <v>341</v>
+        <v>328</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -8020,22 +8035,22 @@
         <v>169</v>
       </c>
       <c r="C26" s="70" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D26" s="70" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="E26" s="70" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="F26" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G26" s="70" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="H26" s="70" t="s">
-        <v>342</v>
+        <v>329</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -8046,22 +8061,22 @@
         <v>169</v>
       </c>
       <c r="C27" s="70" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D27" s="70" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="E27" s="70" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="F27" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G27" s="70" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="H27" s="70" t="s">
-        <v>343</v>
+        <v>330</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -8072,21 +8087,23 @@
         <v>174</v>
       </c>
       <c r="C28" s="70" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="D28" s="70">
         <v>1</v>
       </c>
       <c r="E28" s="70" t="s">
-        <v>376</v>
+        <v>361</v>
       </c>
       <c r="F28" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G28" s="70" t="s">
-        <v>386</v>
-      </c>
-      <c r="H28" s="70"/>
+        <v>371</v>
+      </c>
+      <c r="H28" s="70" t="s">
+        <v>361</v>
+      </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="70" t="s">
@@ -8096,23 +8113,25 @@
         <v>174</v>
       </c>
       <c r="C29" s="70" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="D29" s="70">
         <v>2</v>
       </c>
       <c r="E29" s="70" t="s">
-        <v>377</v>
+        <v>362</v>
       </c>
       <c r="F29" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G29" s="70" t="s">
-        <v>386</v>
-      </c>
-      <c r="H29" s="70"/>
-    </row>
-    <row r="30" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+      <c r="H29" s="70" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="70" t="s">
         <v>244</v>
       </c>
@@ -8120,23 +8139,25 @@
         <v>174</v>
       </c>
       <c r="C30" s="70" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="D30" s="70">
         <v>3</v>
       </c>
       <c r="E30" s="70" t="s">
-        <v>378</v>
+        <v>363</v>
       </c>
       <c r="F30" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G30" s="70" t="s">
-        <v>386</v>
-      </c>
-      <c r="H30" s="70"/>
-    </row>
-    <row r="31" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+      <c r="H30" s="70" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="70" t="s">
         <v>244</v>
       </c>
@@ -8144,23 +8165,25 @@
         <v>174</v>
       </c>
       <c r="C31" s="70" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="D31" s="70">
         <v>4</v>
       </c>
       <c r="E31" s="70" t="s">
-        <v>379</v>
+        <v>364</v>
       </c>
       <c r="F31" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G31" s="70" t="s">
-        <v>386</v>
-      </c>
-      <c r="H31" s="70"/>
-    </row>
-    <row r="32" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+      <c r="H31" s="70" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="70" t="s">
         <v>244</v>
       </c>
@@ -8168,23 +8191,25 @@
         <v>174</v>
       </c>
       <c r="C32" s="70" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="D32" s="70">
         <v>5</v>
       </c>
       <c r="E32" s="70" t="s">
-        <v>380</v>
+        <v>365</v>
       </c>
       <c r="F32" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G32" s="70" t="s">
-        <v>386</v>
-      </c>
-      <c r="H32" s="70"/>
-    </row>
-    <row r="33" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+      <c r="H32" s="70" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="70" t="s">
         <v>244</v>
       </c>
@@ -8192,23 +8217,25 @@
         <v>174</v>
       </c>
       <c r="C33" s="70" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="D33" s="70">
         <v>6</v>
       </c>
       <c r="E33" s="70" t="s">
-        <v>381</v>
+        <v>366</v>
       </c>
       <c r="F33" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G33" s="70" t="s">
-        <v>386</v>
-      </c>
-      <c r="H33" s="70"/>
-    </row>
-    <row r="34" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+      <c r="H33" s="70" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="70" t="s">
         <v>244</v>
       </c>
@@ -8216,23 +8243,25 @@
         <v>174</v>
       </c>
       <c r="C34" s="70" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="D34" s="70">
         <v>7</v>
       </c>
       <c r="E34" s="70" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
       <c r="F34" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G34" s="70" t="s">
-        <v>386</v>
-      </c>
-      <c r="H34" s="70"/>
-    </row>
-    <row r="35" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+      <c r="H34" s="70" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="70" t="s">
         <v>244</v>
       </c>
@@ -8240,23 +8269,25 @@
         <v>174</v>
       </c>
       <c r="C35" s="70" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="D35" s="70">
         <v>8</v>
       </c>
       <c r="E35" s="70" t="s">
-        <v>383</v>
+        <v>368</v>
       </c>
       <c r="F35" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G35" s="70" t="s">
-        <v>386</v>
-      </c>
-      <c r="H35" s="70"/>
-    </row>
-    <row r="36" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+      <c r="H35" s="70" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="70" t="s">
         <v>244</v>
       </c>
@@ -8264,23 +8295,25 @@
         <v>174</v>
       </c>
       <c r="C36" s="70" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="D36" s="70">
         <v>9</v>
       </c>
       <c r="E36" s="70" t="s">
-        <v>384</v>
+        <v>369</v>
       </c>
       <c r="F36" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G36" s="70" t="s">
-        <v>386</v>
-      </c>
-      <c r="H36" s="70"/>
-    </row>
-    <row r="37" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+      <c r="H36" s="70" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="70" t="s">
         <v>244</v>
       </c>
@@ -8288,23 +8321,25 @@
         <v>174</v>
       </c>
       <c r="C37" s="70" t="s">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="D37" s="70">
         <v>10</v>
       </c>
       <c r="E37" s="70" t="s">
-        <v>385</v>
+        <v>370</v>
       </c>
       <c r="F37" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G37" s="70" t="s">
-        <v>386</v>
-      </c>
-      <c r="H37" s="70"/>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+      <c r="H37" s="70" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="70" t="s">
         <v>245</v>
       </c>
@@ -8312,25 +8347,25 @@
         <v>113</v>
       </c>
       <c r="C38" s="70" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="D38" s="70">
         <v>1</v>
       </c>
       <c r="E38" s="70" t="s">
-        <v>275</v>
+        <v>166</v>
       </c>
       <c r="F38" s="70" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="G38" s="70" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="H38" s="70" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="70" t="s">
         <v>245</v>
       </c>
@@ -8338,48 +8373,204 @@
         <v>113</v>
       </c>
       <c r="C39" s="70" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D39" s="70">
         <v>2</v>
       </c>
       <c r="E39" s="70" t="s">
-        <v>279</v>
+        <v>166</v>
       </c>
       <c r="F39" s="70" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="G39" s="70" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="H39" s="70" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="70" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B40" s="70" t="s">
-        <v>247</v>
+        <v>113</v>
       </c>
       <c r="C40" s="70" t="s">
         <v>282</v>
       </c>
       <c r="D40" s="70">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E40" s="70" t="s">
-        <v>283</v>
+        <v>166</v>
       </c>
       <c r="F40" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G40" s="70" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="H40" s="70" t="s">
-        <v>285</v>
+        <v>321</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B41" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C41" s="70" t="s">
+        <v>283</v>
+      </c>
+      <c r="D41" s="70">
+        <v>4</v>
+      </c>
+      <c r="E41" s="70" t="s">
+        <v>166</v>
+      </c>
+      <c r="F41" s="70" t="s">
+        <v>259</v>
+      </c>
+      <c r="G41" s="70" t="s">
+        <v>275</v>
+      </c>
+      <c r="H41" s="70" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B42" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C42" s="70" t="s">
+        <v>267</v>
+      </c>
+      <c r="D42" s="70">
+        <v>5</v>
+      </c>
+      <c r="E42" s="70" t="s">
+        <v>166</v>
+      </c>
+      <c r="F42" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G42" s="70" t="s">
+        <v>268</v>
+      </c>
+      <c r="H42" s="70" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B43" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C43" s="70" t="s">
+        <v>380</v>
+      </c>
+      <c r="D43" s="70">
+        <v>6</v>
+      </c>
+      <c r="E43" s="70" t="s">
+        <v>381</v>
+      </c>
+      <c r="F43" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G43" s="70" t="s">
+        <v>379</v>
+      </c>
+      <c r="H43" s="70" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B44" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C44" s="70" t="s">
+        <v>385</v>
+      </c>
+      <c r="D44" s="70">
+        <v>7</v>
+      </c>
+      <c r="E44" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="F44" s="70" t="s">
+        <v>383</v>
+      </c>
+      <c r="G44" s="70" t="s">
+        <v>384</v>
+      </c>
+      <c r="H44" s="70" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="70" t="s">
+        <v>246</v>
+      </c>
+      <c r="B45" s="70" t="s">
+        <v>247</v>
+      </c>
+      <c r="C45" s="70" t="s">
+        <v>271</v>
+      </c>
+      <c r="D45" s="70">
+        <v>1</v>
+      </c>
+      <c r="E45" s="70" t="s">
+        <v>272</v>
+      </c>
+      <c r="F45" s="70" t="s">
+        <v>259</v>
+      </c>
+      <c r="G45" s="70" t="s">
+        <v>273</v>
+      </c>
+      <c r="H45" s="70" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="70" t="s">
+        <v>246</v>
+      </c>
+      <c r="B46" s="70" t="s">
+        <v>247</v>
+      </c>
+      <c r="C46" s="70" t="s">
+        <v>261</v>
+      </c>
+      <c r="D46" s="70">
+        <v>2</v>
+      </c>
+      <c r="E46" s="70" t="s">
+        <v>388</v>
+      </c>
+      <c r="F46" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G46" s="70" t="s">
+        <v>389</v>
+      </c>
+      <c r="H46" s="70" t="s">
+        <v>390</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: sync updated portfolio checkpoints
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a5263ad85f0b2806/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen HUB\v3\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{5F32698C-664F-4EBB-8172-E004BB472FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BC574CD-1666-4CD6-AC4F-A84C2C262098}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0F9A7E-B711-46B3-9FE6-6F752BA72632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="391">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -964,18 +964,6 @@
     <t>desmistificando_candidaturas</t>
   </si>
   <si>
-    <t>Desmistificando: Vagas publicadas e mercado oculto</t>
-  </si>
-  <si>
-    <t>Revisão e elaboração de CV</t>
-  </si>
-  <si>
-    <t>Preparação para Entrevistas e Networking</t>
-  </si>
-  <si>
-    <t>Feedback Tecnico</t>
-  </si>
-  <si>
     <t>pre_analise_comportamental</t>
   </si>
   <si>
@@ -997,9 +985,6 @@
     <t>A realidade do mercado de trabalho</t>
   </si>
   <si>
-    <t>Preparação de apresentação e pitch em entrevistas</t>
-  </si>
-  <si>
     <t>Avaliação de Perfil Comportamental</t>
   </si>
   <si>
@@ -1075,15 +1060,9 @@
     <t>survey_pdi_fase4</t>
   </si>
   <si>
-    <t>Seleção de recursos e habilidades</t>
-  </si>
-  <si>
     <t>Definição de metas e ciclos</t>
   </si>
   <si>
-    <t>Consolidação de PDI</t>
-  </si>
-  <si>
     <t>master_cv</t>
   </si>
   <si>
@@ -1217,6 +1196,24 @@
   </si>
   <si>
     <t>Avalição de encerramento e consolidação de resultados.</t>
+  </si>
+  <si>
+    <t>Consultoria de Feedback</t>
+  </si>
+  <si>
+    <t>Oportunidades e Mercado Oculto</t>
+  </si>
+  <si>
+    <t>Elaboração de PDI</t>
+  </si>
+  <si>
+    <t>CV e Perfil Profissional</t>
+  </si>
+  <si>
+    <t>Entrevistas e Networking</t>
+  </si>
+  <si>
+    <t>Preparação de apresentação e pitch em entrevistas e reuniões de networking</t>
   </si>
 </sst>
 </file>
@@ -1477,7 +1474,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1717,7 +1714,6 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7478,7 +7474,7 @@
         <v>264</v>
       </c>
       <c r="H4" s="70" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7489,13 +7485,13 @@
         <v>163</v>
       </c>
       <c r="C5" s="70" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D5" s="70">
         <v>1</v>
       </c>
       <c r="E5" s="70" t="s">
-        <v>307</v>
+        <v>386</v>
       </c>
       <c r="F5" s="70" t="s">
         <v>259</v>
@@ -7504,7 +7500,7 @@
         <v>306</v>
       </c>
       <c r="H5" s="70" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7515,22 +7511,22 @@
         <v>163</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="D6" s="70" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>299</v>
+        <v>387</v>
       </c>
       <c r="F6" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G6" s="70" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="H6" s="70" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7541,22 +7537,22 @@
         <v>163</v>
       </c>
       <c r="C7" s="70" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="D7" s="70" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="E7" s="70" t="s">
-        <v>344</v>
+        <v>387</v>
       </c>
       <c r="F7" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G7" s="70" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="H7" s="70" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7567,22 +7563,22 @@
         <v>163</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D8" s="70" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>345</v>
+        <v>387</v>
       </c>
       <c r="F8" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G8" s="70" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="H8" s="70" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7593,22 +7589,22 @@
         <v>163</v>
       </c>
       <c r="C9" s="70" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="D9" s="70" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>346</v>
+        <v>387</v>
       </c>
       <c r="F9" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G9" s="70" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="H9" s="70" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -7619,22 +7615,22 @@
         <v>163</v>
       </c>
       <c r="C10" s="70" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="D10" s="70" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>308</v>
+        <v>388</v>
       </c>
       <c r="F10" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G10" s="70" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="H10" s="70" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7645,22 +7641,22 @@
         <v>163</v>
       </c>
       <c r="C11" s="70" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="D11" s="70" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>308</v>
+        <v>388</v>
       </c>
       <c r="F11" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G11" s="70" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="H11" s="70" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7671,22 +7667,22 @@
         <v>163</v>
       </c>
       <c r="C12" s="70" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="D12" s="70" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>308</v>
+        <v>388</v>
       </c>
       <c r="F12" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G12" s="70" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="H12" s="70" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -7697,22 +7693,22 @@
         <v>163</v>
       </c>
       <c r="C13" s="70" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="D13" s="70">
         <v>4</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>309</v>
+        <v>389</v>
       </c>
       <c r="F13" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G13" s="70" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>318</v>
+        <v>390</v>
       </c>
     </row>
     <row r="14" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7723,22 +7719,22 @@
         <v>163</v>
       </c>
       <c r="C14" s="70" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D14" s="70" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>310</v>
+        <v>385</v>
       </c>
       <c r="F14" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G14" s="70" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="H14" s="70" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -7749,22 +7745,22 @@
         <v>163</v>
       </c>
       <c r="C15" s="70" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="D15" s="70" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>310</v>
+        <v>385</v>
       </c>
       <c r="F15" s="70" t="s">
         <v>259</v>
       </c>
       <c r="G15" s="70" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
       <c r="H15" s="70" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
     </row>
     <row r="16" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7790,7 +7786,7 @@
         <v>266</v>
       </c>
       <c r="H16" s="70" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
     </row>
     <row r="17" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7816,7 +7812,7 @@
         <v>277</v>
       </c>
       <c r="H17" s="70" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -7842,7 +7838,7 @@
         <v>276</v>
       </c>
       <c r="H18" s="70" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="19" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7868,7 +7864,7 @@
         <v>275</v>
       </c>
       <c r="H19" s="70" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
     </row>
     <row r="20" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7894,7 +7890,7 @@
         <v>268</v>
       </c>
       <c r="H20" s="70" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
     </row>
     <row r="21" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7920,7 +7916,7 @@
         <v>284</v>
       </c>
       <c r="H21" s="70" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="22" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7946,7 +7942,7 @@
         <v>287</v>
       </c>
       <c r="H22" s="70" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
     </row>
     <row r="23" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7972,7 +7968,7 @@
         <v>290</v>
       </c>
       <c r="H23" s="70" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -7998,7 +7994,7 @@
         <v>291</v>
       </c>
       <c r="H24" s="70" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -8024,7 +8020,7 @@
         <v>288</v>
       </c>
       <c r="H25" s="70" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -8050,7 +8046,7 @@
         <v>289</v>
       </c>
       <c r="H26" s="70" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -8076,7 +8072,7 @@
         <v>270</v>
       </c>
       <c r="H27" s="70" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -8087,22 +8083,22 @@
         <v>174</v>
       </c>
       <c r="C28" s="70" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D28" s="70">
         <v>1</v>
       </c>
       <c r="E28" s="70" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="F28" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G28" s="70" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H28" s="70" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -8113,22 +8109,22 @@
         <v>174</v>
       </c>
       <c r="C29" s="70" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D29" s="70">
         <v>2</v>
       </c>
       <c r="E29" s="70" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="F29" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G29" s="70" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H29" s="70" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
     </row>
     <row r="30" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -8139,22 +8135,22 @@
         <v>174</v>
       </c>
       <c r="C30" s="70" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D30" s="70">
         <v>3</v>
       </c>
       <c r="E30" s="70" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="F30" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G30" s="70" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H30" s="70" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
     </row>
     <row r="31" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -8165,22 +8161,22 @@
         <v>174</v>
       </c>
       <c r="C31" s="70" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D31" s="70">
         <v>4</v>
       </c>
       <c r="E31" s="70" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="F31" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G31" s="70" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H31" s="70" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
     </row>
     <row r="32" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -8191,22 +8187,22 @@
         <v>174</v>
       </c>
       <c r="C32" s="70" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D32" s="70">
         <v>5</v>
       </c>
       <c r="E32" s="70" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="F32" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G32" s="70" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H32" s="70" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
     </row>
     <row r="33" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -8217,22 +8213,22 @@
         <v>174</v>
       </c>
       <c r="C33" s="70" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D33" s="70">
         <v>6</v>
       </c>
       <c r="E33" s="70" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="F33" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G33" s="70" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H33" s="70" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
     </row>
     <row r="34" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -8243,22 +8239,22 @@
         <v>174</v>
       </c>
       <c r="C34" s="70" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D34" s="70">
         <v>7</v>
       </c>
       <c r="E34" s="70" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
       <c r="F34" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G34" s="70" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H34" s="70" t="s">
-        <v>367</v>
+        <v>360</v>
       </c>
     </row>
     <row r="35" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -8269,22 +8265,22 @@
         <v>174</v>
       </c>
       <c r="C35" s="70" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D35" s="70">
         <v>8</v>
       </c>
       <c r="E35" s="70" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="F35" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G35" s="70" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H35" s="70" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
     </row>
     <row r="36" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -8295,22 +8291,22 @@
         <v>174</v>
       </c>
       <c r="C36" s="70" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D36" s="70">
         <v>9</v>
       </c>
       <c r="E36" s="70" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="F36" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G36" s="70" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H36" s="70" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
     </row>
     <row r="37" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -8321,25 +8317,25 @@
         <v>174</v>
       </c>
       <c r="C37" s="70" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D37" s="70">
         <v>10</v>
       </c>
       <c r="E37" s="70" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="F37" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G37" s="70" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="H37" s="70" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="70" t="s">
         <v>245</v>
       </c>
@@ -8362,10 +8358,10 @@
         <v>266</v>
       </c>
       <c r="H38" s="70" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="70" t="s">
         <v>245</v>
       </c>
@@ -8388,10 +8384,10 @@
         <v>277</v>
       </c>
       <c r="H39" s="70" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="70" t="s">
         <v>245</v>
       </c>
@@ -8414,10 +8410,10 @@
         <v>276</v>
       </c>
       <c r="H40" s="70" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="70" t="s">
         <v>245</v>
       </c>
@@ -8440,10 +8436,10 @@
         <v>275</v>
       </c>
       <c r="H41" s="70" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="70" t="s">
         <v>245</v>
       </c>
@@ -8466,10 +8462,10 @@
         <v>268</v>
       </c>
       <c r="H42" s="70" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="70" t="s">
         <v>245</v>
       </c>
@@ -8477,25 +8473,25 @@
         <v>113</v>
       </c>
       <c r="C43" s="70" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="D43" s="70">
         <v>6</v>
       </c>
       <c r="E43" s="70" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="F43" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G43" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="H43" s="70" t="s">
         <v>379</v>
       </c>
-      <c r="H43" s="70" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="70" t="s">
         <v>245</v>
       </c>
@@ -8503,22 +8499,22 @@
         <v>113</v>
       </c>
       <c r="C44" s="70" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="D44" s="70">
         <v>7</v>
       </c>
       <c r="E44" s="70" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="F44" s="70" t="s">
-        <v>383</v>
+        <v>376</v>
       </c>
       <c r="G44" s="70" t="s">
-        <v>384</v>
+        <v>377</v>
       </c>
       <c r="H44" s="70" t="s">
-        <v>387</v>
+        <v>380</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -8544,7 +8540,7 @@
         <v>273</v>
       </c>
       <c r="H45" s="70" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -8561,16 +8557,16 @@
         <v>2</v>
       </c>
       <c r="E46" s="70" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
       <c r="F46" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G46" s="70" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="H46" s="70" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: set feedback session checkpoint to meeting type and update search keyword filter
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen HUB\v3\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0F9A7E-B711-46B3-9FE6-6F752BA72632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6998232-6CB5-44FF-8B91-5819ECE8A88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7754,7 +7754,7 @@
         <v>385</v>
       </c>
       <c r="F15" s="70" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="G15" s="70" t="s">
         <v>369</v>

</xml_diff>

<commit_message>
Update portfolio_bplen.xlsx with latest changes
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen HUB\v3\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6998232-6CB5-44FF-8B91-5819ECE8A88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A821564-FC28-4246-A95D-B24AE55EE6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Custos gerais" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="396">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -1214,6 +1214,21 @@
   </si>
   <si>
     <t>Preparação de apresentação e pitch em entrevistas e reuniões de networking</t>
+  </si>
+  <si>
+    <t>1.1</t>
+  </si>
+  <si>
+    <t>1.2</t>
+  </si>
+  <si>
+    <t>1.3</t>
+  </si>
+  <si>
+    <t>1.4</t>
+  </si>
+  <si>
+    <t>1.5</t>
   </si>
 </sst>
 </file>
@@ -8345,8 +8360,8 @@
       <c r="C38" s="70" t="s">
         <v>265</v>
       </c>
-      <c r="D38" s="70">
-        <v>1</v>
+      <c r="D38" s="70" t="s">
+        <v>391</v>
       </c>
       <c r="E38" s="70" t="s">
         <v>166</v>
@@ -8371,8 +8386,8 @@
       <c r="C39" s="70" t="s">
         <v>281</v>
       </c>
-      <c r="D39" s="70">
-        <v>2</v>
+      <c r="D39" s="70" t="s">
+        <v>392</v>
       </c>
       <c r="E39" s="70" t="s">
         <v>166</v>
@@ -8397,8 +8412,8 @@
       <c r="C40" s="70" t="s">
         <v>282</v>
       </c>
-      <c r="D40" s="70">
-        <v>3</v>
+      <c r="D40" s="70" t="s">
+        <v>393</v>
       </c>
       <c r="E40" s="70" t="s">
         <v>166</v>
@@ -8423,8 +8438,8 @@
       <c r="C41" s="70" t="s">
         <v>283</v>
       </c>
-      <c r="D41" s="70">
-        <v>4</v>
+      <c r="D41" s="70" t="s">
+        <v>394</v>
       </c>
       <c r="E41" s="70" t="s">
         <v>166</v>
@@ -8449,8 +8464,8 @@
       <c r="C42" s="70" t="s">
         <v>267</v>
       </c>
-      <c r="D42" s="70">
-        <v>5</v>
+      <c r="D42" s="70" t="s">
+        <v>395</v>
       </c>
       <c r="E42" s="70" t="s">
         <v>166</v>

</xml_diff>

<commit_message>
chore: Update portfolio payload after excel edits
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen HUB\v3\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A821564-FC28-4246-A95D-B24AE55EE6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBB1ABB-CE59-45C8-9E04-1D92F03E4F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="400">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -1165,27 +1165,9 @@
     <t>agendar-sessao-mentocoach</t>
   </si>
   <si>
-    <t>Sessões de MentoCoach</t>
-  </si>
-  <si>
-    <t>MentoCoach Dashboard</t>
-  </si>
-  <si>
-    <t>dashboard</t>
-  </si>
-  <si>
-    <t>mentocoach-dashboard</t>
-  </si>
-  <si>
-    <t>realizar-mentocoach-dashboard</t>
-  </si>
-  <si>
     <t>Sessão de MentoCoach</t>
   </si>
   <si>
-    <t>Acompanhamento do Progresso</t>
-  </si>
-  <si>
     <t>Sessão de Offboarding</t>
   </si>
   <si>
@@ -1229,6 +1211,36 @@
   </si>
   <si>
     <t>1.5</t>
+  </si>
+  <si>
+    <t>1ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>2ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>3ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>4ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>5ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>6ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>7ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>8ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>9ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>10ª Sessão de MentoCoach</t>
   </si>
 </sst>
 </file>
@@ -7384,7 +7396,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9" style="70"/>
@@ -7506,7 +7518,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="70" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="F5" s="70" t="s">
         <v>259</v>
@@ -7532,7 +7544,7 @@
         <v>327</v>
       </c>
       <c r="E6" s="70" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="F6" s="70" t="s">
         <v>259</v>
@@ -7558,7 +7570,7 @@
         <v>330</v>
       </c>
       <c r="E7" s="70" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="F7" s="70" t="s">
         <v>259</v>
@@ -7584,7 +7596,7 @@
         <v>334</v>
       </c>
       <c r="E8" s="70" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="F8" s="70" t="s">
         <v>259</v>
@@ -7610,7 +7622,7 @@
         <v>337</v>
       </c>
       <c r="E9" s="70" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="F9" s="70" t="s">
         <v>259</v>
@@ -7636,7 +7648,7 @@
         <v>344</v>
       </c>
       <c r="E10" s="70" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="F10" s="70" t="s">
         <v>259</v>
@@ -7662,7 +7674,7 @@
         <v>345</v>
       </c>
       <c r="E11" s="70" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="F11" s="70" t="s">
         <v>259</v>
@@ -7688,7 +7700,7 @@
         <v>346</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="F12" s="70" t="s">
         <v>259</v>
@@ -7714,7 +7726,7 @@
         <v>4</v>
       </c>
       <c r="E13" s="70" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="F13" s="70" t="s">
         <v>259</v>
@@ -7723,7 +7735,7 @@
         <v>365</v>
       </c>
       <c r="H13" s="70" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
     </row>
     <row r="14" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -7740,7 +7752,7 @@
         <v>310</v>
       </c>
       <c r="E14" s="70" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="F14" s="70" t="s">
         <v>259</v>
@@ -7766,7 +7778,7 @@
         <v>311</v>
       </c>
       <c r="E15" s="70" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="F15" s="70" t="s">
         <v>263</v>
@@ -8361,7 +8373,7 @@
         <v>265</v>
       </c>
       <c r="D38" s="70" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="E38" s="70" t="s">
         <v>166</v>
@@ -8387,7 +8399,7 @@
         <v>281</v>
       </c>
       <c r="D39" s="70" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="E39" s="70" t="s">
         <v>166</v>
@@ -8413,7 +8425,7 @@
         <v>282</v>
       </c>
       <c r="D40" s="70" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="E40" s="70" t="s">
         <v>166</v>
@@ -8439,7 +8451,7 @@
         <v>283</v>
       </c>
       <c r="D41" s="70" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="E41" s="70" t="s">
         <v>166</v>
@@ -8465,7 +8477,7 @@
         <v>267</v>
       </c>
       <c r="D42" s="70" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="E42" s="70" t="s">
         <v>166</v>
@@ -8491,10 +8503,10 @@
         <v>373</v>
       </c>
       <c r="D43" s="70">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E43" s="70" t="s">
-        <v>374</v>
+        <v>390</v>
       </c>
       <c r="F43" s="70" t="s">
         <v>263</v>
@@ -8503,7 +8515,7 @@
         <v>372</v>
       </c>
       <c r="H43" s="70" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="44" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
@@ -8514,74 +8526,282 @@
         <v>113</v>
       </c>
       <c r="C44" s="70" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="D44" s="70">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E44" s="70" t="s">
-        <v>375</v>
+        <v>391</v>
       </c>
       <c r="F44" s="70" t="s">
-        <v>376</v>
+        <v>263</v>
       </c>
       <c r="G44" s="70" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="H44" s="70" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="70" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B45" s="70" t="s">
-        <v>247</v>
+        <v>113</v>
       </c>
       <c r="C45" s="70" t="s">
-        <v>271</v>
+        <v>373</v>
       </c>
       <c r="D45" s="70">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E45" s="70" t="s">
-        <v>272</v>
+        <v>392</v>
       </c>
       <c r="F45" s="70" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="G45" s="70" t="s">
-        <v>273</v>
+        <v>372</v>
       </c>
       <c r="H45" s="70" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="70" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B46" s="70" t="s">
-        <v>247</v>
+        <v>113</v>
       </c>
       <c r="C46" s="70" t="s">
-        <v>261</v>
+        <v>373</v>
       </c>
       <c r="D46" s="70">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E46" s="70" t="s">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="F46" s="70" t="s">
         <v>263</v>
       </c>
       <c r="G46" s="70" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="H46" s="70" t="s">
-        <v>383</v>
+        <v>374</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B47" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C47" s="70" t="s">
+        <v>373</v>
+      </c>
+      <c r="D47" s="70">
+        <v>6</v>
+      </c>
+      <c r="E47" s="70" t="s">
+        <v>394</v>
+      </c>
+      <c r="F47" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G47" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="H47" s="70" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B48" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C48" s="70" t="s">
+        <v>373</v>
+      </c>
+      <c r="D48" s="70">
+        <v>7</v>
+      </c>
+      <c r="E48" s="70" t="s">
+        <v>395</v>
+      </c>
+      <c r="F48" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G48" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="H48" s="70" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B49" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C49" s="70" t="s">
+        <v>373</v>
+      </c>
+      <c r="D49" s="70">
+        <v>8</v>
+      </c>
+      <c r="E49" s="70" t="s">
+        <v>396</v>
+      </c>
+      <c r="F49" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G49" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="H49" s="70" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B50" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C50" s="70" t="s">
+        <v>373</v>
+      </c>
+      <c r="D50" s="70">
+        <v>9</v>
+      </c>
+      <c r="E50" s="70" t="s">
+        <v>397</v>
+      </c>
+      <c r="F50" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G50" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="H50" s="70" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B51" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C51" s="70" t="s">
+        <v>373</v>
+      </c>
+      <c r="D51" s="70">
+        <v>10</v>
+      </c>
+      <c r="E51" s="70" t="s">
+        <v>398</v>
+      </c>
+      <c r="F51" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G51" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="H51" s="70" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" s="70" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="70" t="s">
+        <v>245</v>
+      </c>
+      <c r="B52" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="C52" s="70" t="s">
+        <v>373</v>
+      </c>
+      <c r="D52" s="70">
+        <v>11</v>
+      </c>
+      <c r="E52" s="70" t="s">
+        <v>399</v>
+      </c>
+      <c r="F52" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G52" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="H52" s="70" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="70" t="s">
+        <v>246</v>
+      </c>
+      <c r="B53" s="70" t="s">
+        <v>247</v>
+      </c>
+      <c r="C53" s="70" t="s">
+        <v>271</v>
+      </c>
+      <c r="D53" s="70">
+        <v>1</v>
+      </c>
+      <c r="E53" s="70" t="s">
+        <v>272</v>
+      </c>
+      <c r="F53" s="70" t="s">
+        <v>259</v>
+      </c>
+      <c r="G53" s="70" t="s">
+        <v>273</v>
+      </c>
+      <c r="H53" s="70" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="70" t="s">
+        <v>246</v>
+      </c>
+      <c r="B54" s="70" t="s">
+        <v>247</v>
+      </c>
+      <c r="C54" s="70" t="s">
+        <v>261</v>
+      </c>
+      <c r="D54" s="70">
+        <v>2</v>
+      </c>
+      <c r="E54" s="70" t="s">
+        <v>375</v>
+      </c>
+      <c r="F54" s="70" t="s">
+        <v>263</v>
+      </c>
+      <c r="G54" s="70" t="s">
+        <v>376</v>
+      </c>
+      <c r="H54" s="70" t="s">
+        <v>377</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data(portfolio): aba Atributos preenchida + payload regenerado (pre-Sync) (#34)
Commita a fonte (xlsx, aba Atributos preenchida pela Gestora e validada contra
ACCESS-MODEL-DESIGN.md secao 3.1) e o portfolio_payload.json regenerado: os 12
produtos ganham escopo/concedeSelo/preRequisitos/libera. Validacao estrita por
diff: zero mudanca em campos existentes; BPL-PAC-JR = public + concedeSelo
false + libera [BPL-001].

Este merge NAO toca o Firestore. A virada acontece no clique de "Sincronizar
Portfolio" no admin (le o payload deployado) — e ai o A2 ativa: junior e
posicionamento param de conceder o selo de membro.

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen HUB\v3\portfolio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen_HUB\Dev\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBB1ABB-CE59-45C8-9E04-1D92F03E4F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3B1262-7FC5-4499-B50A-7EF50E1C7BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="728" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Custos gerais" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="Metas" sheetId="7" r:id="rId7"/>
     <sheet name="Jornada" sheetId="8" r:id="rId8"/>
     <sheet name="Checkpoints" sheetId="9" r:id="rId9"/>
+    <sheet name="Atributos" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="434">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -1241,6 +1242,108 @@
   </si>
   <si>
     <t>10ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>serviceCode</t>
+  </si>
+  <si>
+    <t>serviceName</t>
+  </si>
+  <si>
+    <t>escopo</t>
+  </si>
+  <si>
+    <t>concedeSelo</t>
+  </si>
+  <si>
+    <t>preReqModo</t>
+  </si>
+  <si>
+    <t>preReqEtapas</t>
+  </si>
+  <si>
+    <t>libera</t>
+  </si>
+  <si>
+    <t>sku</t>
+  </si>
+  <si>
+    <t>nbs</t>
+  </si>
+  <si>
+    <t>naturezaOperacao</t>
+  </si>
+  <si>
+    <t>descricaoFiscal</t>
+  </si>
+  <si>
+    <t>public</t>
+  </si>
+  <si>
+    <t>FALSE</t>
+  </si>
+  <si>
+    <t>nenhum</t>
+  </si>
+  <si>
+    <t>member</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>todos</t>
+  </si>
+  <si>
+    <t>Gestão e Desenv. de Carreira</t>
+  </si>
+  <si>
+    <t>qualquer</t>
+  </si>
+  <si>
+    <t>BPL-004,BPL-005</t>
+  </si>
+  <si>
+    <t>BPL-PAC-JR</t>
+  </si>
+  <si>
+    <t>Pacote Junior</t>
+  </si>
+  <si>
+    <t>BPL-PAC-PL</t>
+  </si>
+  <si>
+    <t>Pacote Pleno</t>
+  </si>
+  <si>
+    <t>BPL-001,BPL-002</t>
+  </si>
+  <si>
+    <t>BPL-PAC-SR</t>
+  </si>
+  <si>
+    <t>Pacote Senior</t>
+  </si>
+  <si>
+    <t>BPL-001,BPL-002,BPL-003</t>
+  </si>
+  <si>
+    <t>BPL-PAC-LD</t>
+  </si>
+  <si>
+    <t>Pacote Líder</t>
+  </si>
+  <si>
+    <t>BPL-001,BPL-002,BPL-003,BPL-004</t>
+  </si>
+  <si>
+    <t>BPL-PAC-EB</t>
+  </si>
+  <si>
+    <t>Pacote Embaixador</t>
+  </si>
+  <si>
+    <t>BPL-001,BPL-002,BPL-003,BPL-004,BPL-005</t>
   </si>
 </sst>
 </file>
@@ -1501,7 +1604,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1739,6 +1842,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
@@ -2244,6 +2353,293 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{403060E9-08D3-4832-A865-DE6A12F50842}">
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.375" style="103" customWidth="1"/>
+    <col min="2" max="2" width="15.125" style="103" customWidth="1"/>
+    <col min="3" max="3" width="9" style="103"/>
+    <col min="4" max="4" width="10.75" style="103" customWidth="1"/>
+    <col min="5" max="5" width="11.25" style="103" customWidth="1"/>
+    <col min="6" max="6" width="13.125" style="103" customWidth="1"/>
+    <col min="7" max="7" width="17.25" style="103" customWidth="1"/>
+    <col min="8" max="9" width="9" style="103"/>
+    <col min="10" max="10" width="18.25" style="103" customWidth="1"/>
+    <col min="11" max="11" width="17.75" style="103" customWidth="1"/>
+    <col min="12" max="16384" width="9" style="103"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="104" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="104" t="s">
+        <v>400</v>
+      </c>
+      <c r="B1" s="104" t="s">
+        <v>401</v>
+      </c>
+      <c r="C1" s="104" t="s">
+        <v>402</v>
+      </c>
+      <c r="D1" s="104" t="s">
+        <v>403</v>
+      </c>
+      <c r="E1" s="104" t="s">
+        <v>404</v>
+      </c>
+      <c r="F1" s="104" t="s">
+        <v>405</v>
+      </c>
+      <c r="G1" s="104" t="s">
+        <v>406</v>
+      </c>
+      <c r="H1" s="104" t="s">
+        <v>407</v>
+      </c>
+      <c r="I1" s="104" t="s">
+        <v>408</v>
+      </c>
+      <c r="J1" s="104" t="s">
+        <v>409</v>
+      </c>
+      <c r="K1" s="104" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="103" t="s">
+        <v>241</v>
+      </c>
+      <c r="B2" s="103" t="s">
+        <v>163</v>
+      </c>
+      <c r="C2" s="103" t="s">
+        <v>411</v>
+      </c>
+      <c r="D2" s="103" t="s">
+        <v>412</v>
+      </c>
+      <c r="E2" s="103" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="103" t="s">
+        <v>239</v>
+      </c>
+      <c r="B3" s="103" t="s">
+        <v>240</v>
+      </c>
+      <c r="C3" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D3" s="103" t="s">
+        <v>412</v>
+      </c>
+      <c r="E3" s="103" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="103" t="s">
+        <v>242</v>
+      </c>
+      <c r="B4" s="103" t="s">
+        <v>166</v>
+      </c>
+      <c r="C4" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D4" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E4" s="103" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="103" t="s">
+        <v>243</v>
+      </c>
+      <c r="B5" s="103" t="s">
+        <v>169</v>
+      </c>
+      <c r="C5" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D5" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E5" s="103" t="s">
+        <v>416</v>
+      </c>
+      <c r="F5" s="103" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="103" t="s">
+        <v>244</v>
+      </c>
+      <c r="B6" s="103" t="s">
+        <v>417</v>
+      </c>
+      <c r="C6" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D6" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E6" s="103" t="s">
+        <v>416</v>
+      </c>
+      <c r="F6" s="103" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="103" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" s="103" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D7" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E7" s="103" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="103" t="s">
+        <v>246</v>
+      </c>
+      <c r="B8" s="103" t="s">
+        <v>247</v>
+      </c>
+      <c r="C8" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D8" s="103" t="s">
+        <v>412</v>
+      </c>
+      <c r="E8" s="103" t="s">
+        <v>418</v>
+      </c>
+      <c r="F8" s="103" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="103" t="s">
+        <v>420</v>
+      </c>
+      <c r="B9" s="103" t="s">
+        <v>421</v>
+      </c>
+      <c r="C9" s="103" t="s">
+        <v>411</v>
+      </c>
+      <c r="D9" s="103" t="s">
+        <v>412</v>
+      </c>
+      <c r="E9" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="G9" s="103" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="103" t="s">
+        <v>422</v>
+      </c>
+      <c r="B10" s="103" t="s">
+        <v>423</v>
+      </c>
+      <c r="C10" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D10" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E10" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="G10" s="103" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="103" t="s">
+        <v>425</v>
+      </c>
+      <c r="B11" s="103" t="s">
+        <v>426</v>
+      </c>
+      <c r="C11" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D11" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E11" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="G11" s="103" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="103" t="s">
+        <v>428</v>
+      </c>
+      <c r="B12" s="103" t="s">
+        <v>429</v>
+      </c>
+      <c r="C12" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D12" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E12" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="G12" s="103" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="103" t="s">
+        <v>431</v>
+      </c>
+      <c r="B13" s="103" t="s">
+        <v>432</v>
+      </c>
+      <c r="C13" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D13" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E13" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="G13" s="103" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:E27"/>
@@ -5264,13 +5660,13 @@
     </row>
     <row r="15" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="103" t="s">
+      <c r="B16" s="105" t="s">
         <v>198</v>
       </c>
-      <c r="C16" s="104"/>
-      <c r="D16" s="104"/>
-      <c r="E16" s="104"/>
-      <c r="F16" s="104"/>
+      <c r="C16" s="106"/>
+      <c r="D16" s="106"/>
+      <c r="E16" s="106"/>
+      <c r="F16" s="106"/>
     </row>
     <row r="17" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="61" t="s">
@@ -5492,13 +5888,13 @@
     </row>
     <row r="32" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="103" t="s">
+      <c r="B33" s="105" t="s">
         <v>216</v>
       </c>
-      <c r="C33" s="104"/>
-      <c r="D33" s="104"/>
-      <c r="E33" s="104"/>
-      <c r="F33" s="104"/>
+      <c r="C33" s="106"/>
+      <c r="D33" s="106"/>
+      <c r="E33" s="106"/>
+      <c r="F33" s="106"/>
     </row>
     <row r="34" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="61" t="s">
@@ -5800,13 +6196,13 @@
     </row>
     <row r="54" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="103" t="s">
+      <c r="B55" s="105" t="s">
         <v>224</v>
       </c>
-      <c r="C55" s="104"/>
-      <c r="D55" s="104"/>
-      <c r="E55" s="104"/>
-      <c r="F55" s="104"/>
+      <c r="C55" s="106"/>
+      <c r="D55" s="106"/>
+      <c r="E55" s="106"/>
+      <c r="F55" s="106"/>
     </row>
     <row r="56" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="61" t="s">
@@ -6127,13 +6523,13 @@
       </c>
     </row>
     <row r="78" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="103" t="s">
+      <c r="B78" s="105" t="s">
         <v>228</v>
       </c>
-      <c r="C78" s="104"/>
-      <c r="D78" s="104"/>
-      <c r="E78" s="104"/>
-      <c r="F78" s="104"/>
+      <c r="C78" s="106"/>
+      <c r="D78" s="106"/>
+      <c r="E78" s="106"/>
+      <c r="F78" s="106"/>
     </row>
     <row r="79" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="61" t="s">
@@ -6487,13 +6883,13 @@
     </row>
     <row r="101" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B102" s="103" t="s">
+      <c r="B102" s="105" t="s">
         <v>232</v>
       </c>
-      <c r="C102" s="104"/>
-      <c r="D102" s="104"/>
-      <c r="E102" s="104"/>
-      <c r="F102" s="104"/>
+      <c r="C102" s="106"/>
+      <c r="D102" s="106"/>
+      <c r="E102" s="106"/>
+      <c r="F102" s="106"/>
     </row>
     <row r="103" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="61" t="s">

</xml_diff>

<commit_message>
data(portfolio): aba Atributos preenchida + payload regenerado (pre-Sync)
Commita a fonte (xlsx, aba Atributos preenchida pela Gestora e validada contra
ACCESS-MODEL-DESIGN.md secao 3.1) e o portfolio_payload.json regenerado: os 12
produtos ganham escopo/concedeSelo/preRequisitos/libera. Validacao estrita por
diff: zero mudanca em campos existentes; BPL-PAC-JR = public + concedeSelo
false + libera [BPL-001].

Este merge NAO toca o Firestore. A virada acontece no clique de "Sincronizar
Portfolio" no admin (le o payload deployado) — e ai o A2 ativa: junior e
posicionamento param de conceder o selo de membro.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen HUB\v3\portfolio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen_HUB\Dev\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBB1ABB-CE59-45C8-9E04-1D92F03E4F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3B1262-7FC5-4499-B50A-7EF50E1C7BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="728" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Custos gerais" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="Metas" sheetId="7" r:id="rId7"/>
     <sheet name="Jornada" sheetId="8" r:id="rId8"/>
     <sheet name="Checkpoints" sheetId="9" r:id="rId9"/>
+    <sheet name="Atributos" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="434">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -1241,6 +1242,108 @@
   </si>
   <si>
     <t>10ª Sessão de MentoCoach</t>
+  </si>
+  <si>
+    <t>serviceCode</t>
+  </si>
+  <si>
+    <t>serviceName</t>
+  </si>
+  <si>
+    <t>escopo</t>
+  </si>
+  <si>
+    <t>concedeSelo</t>
+  </si>
+  <si>
+    <t>preReqModo</t>
+  </si>
+  <si>
+    <t>preReqEtapas</t>
+  </si>
+  <si>
+    <t>libera</t>
+  </si>
+  <si>
+    <t>sku</t>
+  </si>
+  <si>
+    <t>nbs</t>
+  </si>
+  <si>
+    <t>naturezaOperacao</t>
+  </si>
+  <si>
+    <t>descricaoFiscal</t>
+  </si>
+  <si>
+    <t>public</t>
+  </si>
+  <si>
+    <t>FALSE</t>
+  </si>
+  <si>
+    <t>nenhum</t>
+  </si>
+  <si>
+    <t>member</t>
+  </si>
+  <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>todos</t>
+  </si>
+  <si>
+    <t>Gestão e Desenv. de Carreira</t>
+  </si>
+  <si>
+    <t>qualquer</t>
+  </si>
+  <si>
+    <t>BPL-004,BPL-005</t>
+  </si>
+  <si>
+    <t>BPL-PAC-JR</t>
+  </si>
+  <si>
+    <t>Pacote Junior</t>
+  </si>
+  <si>
+    <t>BPL-PAC-PL</t>
+  </si>
+  <si>
+    <t>Pacote Pleno</t>
+  </si>
+  <si>
+    <t>BPL-001,BPL-002</t>
+  </si>
+  <si>
+    <t>BPL-PAC-SR</t>
+  </si>
+  <si>
+    <t>Pacote Senior</t>
+  </si>
+  <si>
+    <t>BPL-001,BPL-002,BPL-003</t>
+  </si>
+  <si>
+    <t>BPL-PAC-LD</t>
+  </si>
+  <si>
+    <t>Pacote Líder</t>
+  </si>
+  <si>
+    <t>BPL-001,BPL-002,BPL-003,BPL-004</t>
+  </si>
+  <si>
+    <t>BPL-PAC-EB</t>
+  </si>
+  <si>
+    <t>Pacote Embaixador</t>
+  </si>
+  <si>
+    <t>BPL-001,BPL-002,BPL-003,BPL-004,BPL-005</t>
   </si>
 </sst>
 </file>
@@ -1501,7 +1604,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1739,6 +1842,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
@@ -2244,6 +2353,293 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{403060E9-08D3-4832-A865-DE6A12F50842}">
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.375" style="103" customWidth="1"/>
+    <col min="2" max="2" width="15.125" style="103" customWidth="1"/>
+    <col min="3" max="3" width="9" style="103"/>
+    <col min="4" max="4" width="10.75" style="103" customWidth="1"/>
+    <col min="5" max="5" width="11.25" style="103" customWidth="1"/>
+    <col min="6" max="6" width="13.125" style="103" customWidth="1"/>
+    <col min="7" max="7" width="17.25" style="103" customWidth="1"/>
+    <col min="8" max="9" width="9" style="103"/>
+    <col min="10" max="10" width="18.25" style="103" customWidth="1"/>
+    <col min="11" max="11" width="17.75" style="103" customWidth="1"/>
+    <col min="12" max="16384" width="9" style="103"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="104" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="104" t="s">
+        <v>400</v>
+      </c>
+      <c r="B1" s="104" t="s">
+        <v>401</v>
+      </c>
+      <c r="C1" s="104" t="s">
+        <v>402</v>
+      </c>
+      <c r="D1" s="104" t="s">
+        <v>403</v>
+      </c>
+      <c r="E1" s="104" t="s">
+        <v>404</v>
+      </c>
+      <c r="F1" s="104" t="s">
+        <v>405</v>
+      </c>
+      <c r="G1" s="104" t="s">
+        <v>406</v>
+      </c>
+      <c r="H1" s="104" t="s">
+        <v>407</v>
+      </c>
+      <c r="I1" s="104" t="s">
+        <v>408</v>
+      </c>
+      <c r="J1" s="104" t="s">
+        <v>409</v>
+      </c>
+      <c r="K1" s="104" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="103" t="s">
+        <v>241</v>
+      </c>
+      <c r="B2" s="103" t="s">
+        <v>163</v>
+      </c>
+      <c r="C2" s="103" t="s">
+        <v>411</v>
+      </c>
+      <c r="D2" s="103" t="s">
+        <v>412</v>
+      </c>
+      <c r="E2" s="103" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="103" t="s">
+        <v>239</v>
+      </c>
+      <c r="B3" s="103" t="s">
+        <v>240</v>
+      </c>
+      <c r="C3" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D3" s="103" t="s">
+        <v>412</v>
+      </c>
+      <c r="E3" s="103" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="103" t="s">
+        <v>242</v>
+      </c>
+      <c r="B4" s="103" t="s">
+        <v>166</v>
+      </c>
+      <c r="C4" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D4" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E4" s="103" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="103" t="s">
+        <v>243</v>
+      </c>
+      <c r="B5" s="103" t="s">
+        <v>169</v>
+      </c>
+      <c r="C5" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D5" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E5" s="103" t="s">
+        <v>416</v>
+      </c>
+      <c r="F5" s="103" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="103" t="s">
+        <v>244</v>
+      </c>
+      <c r="B6" s="103" t="s">
+        <v>417</v>
+      </c>
+      <c r="C6" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D6" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E6" s="103" t="s">
+        <v>416</v>
+      </c>
+      <c r="F6" s="103" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="103" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" s="103" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D7" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E7" s="103" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="103" t="s">
+        <v>246</v>
+      </c>
+      <c r="B8" s="103" t="s">
+        <v>247</v>
+      </c>
+      <c r="C8" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D8" s="103" t="s">
+        <v>412</v>
+      </c>
+      <c r="E8" s="103" t="s">
+        <v>418</v>
+      </c>
+      <c r="F8" s="103" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="103" t="s">
+        <v>420</v>
+      </c>
+      <c r="B9" s="103" t="s">
+        <v>421</v>
+      </c>
+      <c r="C9" s="103" t="s">
+        <v>411</v>
+      </c>
+      <c r="D9" s="103" t="s">
+        <v>412</v>
+      </c>
+      <c r="E9" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="G9" s="103" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="103" t="s">
+        <v>422</v>
+      </c>
+      <c r="B10" s="103" t="s">
+        <v>423</v>
+      </c>
+      <c r="C10" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D10" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E10" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="G10" s="103" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="103" t="s">
+        <v>425</v>
+      </c>
+      <c r="B11" s="103" t="s">
+        <v>426</v>
+      </c>
+      <c r="C11" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D11" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E11" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="G11" s="103" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="103" t="s">
+        <v>428</v>
+      </c>
+      <c r="B12" s="103" t="s">
+        <v>429</v>
+      </c>
+      <c r="C12" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D12" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E12" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="G12" s="103" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="103" t="s">
+        <v>431</v>
+      </c>
+      <c r="B13" s="103" t="s">
+        <v>432</v>
+      </c>
+      <c r="C13" s="103" t="s">
+        <v>414</v>
+      </c>
+      <c r="D13" s="103" t="s">
+        <v>415</v>
+      </c>
+      <c r="E13" s="103" t="s">
+        <v>413</v>
+      </c>
+      <c r="G13" s="103" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:E27"/>
@@ -5264,13 +5660,13 @@
     </row>
     <row r="15" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="2:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="103" t="s">
+      <c r="B16" s="105" t="s">
         <v>198</v>
       </c>
-      <c r="C16" s="104"/>
-      <c r="D16" s="104"/>
-      <c r="E16" s="104"/>
-      <c r="F16" s="104"/>
+      <c r="C16" s="106"/>
+      <c r="D16" s="106"/>
+      <c r="E16" s="106"/>
+      <c r="F16" s="106"/>
     </row>
     <row r="17" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="61" t="s">
@@ -5492,13 +5888,13 @@
     </row>
     <row r="32" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="103" t="s">
+      <c r="B33" s="105" t="s">
         <v>216</v>
       </c>
-      <c r="C33" s="104"/>
-      <c r="D33" s="104"/>
-      <c r="E33" s="104"/>
-      <c r="F33" s="104"/>
+      <c r="C33" s="106"/>
+      <c r="D33" s="106"/>
+      <c r="E33" s="106"/>
+      <c r="F33" s="106"/>
     </row>
     <row r="34" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="61" t="s">
@@ -5800,13 +6196,13 @@
     </row>
     <row r="54" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="103" t="s">
+      <c r="B55" s="105" t="s">
         <v>224</v>
       </c>
-      <c r="C55" s="104"/>
-      <c r="D55" s="104"/>
-      <c r="E55" s="104"/>
-      <c r="F55" s="104"/>
+      <c r="C55" s="106"/>
+      <c r="D55" s="106"/>
+      <c r="E55" s="106"/>
+      <c r="F55" s="106"/>
     </row>
     <row r="56" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="61" t="s">
@@ -6127,13 +6523,13 @@
       </c>
     </row>
     <row r="78" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="103" t="s">
+      <c r="B78" s="105" t="s">
         <v>228</v>
       </c>
-      <c r="C78" s="104"/>
-      <c r="D78" s="104"/>
-      <c r="E78" s="104"/>
-      <c r="F78" s="104"/>
+      <c r="C78" s="106"/>
+      <c r="D78" s="106"/>
+      <c r="E78" s="106"/>
+      <c r="F78" s="106"/>
     </row>
     <row r="79" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="61" t="s">
@@ -6487,13 +6883,13 @@
     </row>
     <row r="101" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="102" spans="2:6" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B102" s="103" t="s">
+      <c r="B102" s="105" t="s">
         <v>232</v>
       </c>
-      <c r="C102" s="104"/>
-      <c r="D102" s="104"/>
-      <c r="E102" s="104"/>
-      <c r="F102" s="104"/>
+      <c r="C102" s="106"/>
+      <c r="D102" s="106"/>
+      <c r="E102" s="106"/>
+      <c r="F102" s="106"/>
     </row>
     <row r="103" spans="2:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="61" t="s">

</xml_diff>

<commit_message>
data(portfolio): onboarding como pre-requisito + pacotes liberam BPL-000 (#36)
Revisao da Gestora na aba Atributos (pos-B2): BPL-000 vira pre-req de
analise/plano/GDC/mentocoach e os pacotes pleno..embaixador liberam BPL-000.
Primeira mudanca de regra feita puramente por dado — zero codigo; o motor da
Fase B2 aplica. Validado por diff: so preRequisitos/libera mudaram.

Vigora no proximo clique de Sincronizar Portfolio.

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen_HUB\Dev\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3B1262-7FC5-4499-B50A-7EF50E1C7BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5467C438-FCE7-487F-BF5F-135A45D3C8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="728" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="436">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -1316,34 +1316,40 @@
     <t>Pacote Pleno</t>
   </si>
   <si>
-    <t>BPL-001,BPL-002</t>
-  </si>
-  <si>
     <t>BPL-PAC-SR</t>
   </si>
   <si>
     <t>Pacote Senior</t>
   </si>
   <si>
-    <t>BPL-001,BPL-002,BPL-003</t>
-  </si>
-  <si>
     <t>BPL-PAC-LD</t>
   </si>
   <si>
     <t>Pacote Líder</t>
   </si>
   <si>
-    <t>BPL-001,BPL-002,BPL-003,BPL-004</t>
-  </si>
-  <si>
     <t>BPL-PAC-EB</t>
   </si>
   <si>
     <t>Pacote Embaixador</t>
   </si>
   <si>
-    <t>BPL-001,BPL-002,BPL-003,BPL-004,BPL-005</t>
+    <t>BPL-000,BPL-002</t>
+  </si>
+  <si>
+    <t>BPL-000,BPL-003</t>
+  </si>
+  <si>
+    <t>BPL-000,BPL-001,BPL-002</t>
+  </si>
+  <si>
+    <t>BPL-000,BPL-001,BPL-002,BPL-003</t>
+  </si>
+  <si>
+    <t>BPL-000,BPL-001,BPL-002,BPL-003,BPL-004</t>
+  </si>
+  <si>
+    <t>BPL-000,BPL-001,BPL-002,BPL-003,BPL-004,BPL-005</t>
   </si>
 </sst>
 </file>
@@ -2454,7 +2460,10 @@
         <v>415</v>
       </c>
       <c r="E4" s="103" t="s">
-        <v>413</v>
+        <v>416</v>
+      </c>
+      <c r="F4" s="103" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2474,7 +2483,7 @@
         <v>416</v>
       </c>
       <c r="F5" s="103" t="s">
-        <v>242</v>
+        <v>430</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2494,7 +2503,7 @@
         <v>416</v>
       </c>
       <c r="F6" s="103" t="s">
-        <v>243</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2511,7 +2520,10 @@
         <v>415</v>
       </c>
       <c r="E7" s="103" t="s">
-        <v>413</v>
+        <v>416</v>
+      </c>
+      <c r="F7" s="103" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2571,15 +2583,15 @@
         <v>413</v>
       </c>
       <c r="G10" s="103" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="103" t="s">
+        <v>424</v>
+      </c>
+      <c r="B11" s="103" t="s">
         <v>425</v>
-      </c>
-      <c r="B11" s="103" t="s">
-        <v>426</v>
       </c>
       <c r="C11" s="103" t="s">
         <v>414</v>
@@ -2591,15 +2603,15 @@
         <v>413</v>
       </c>
       <c r="G11" s="103" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="103" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B12" s="103" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C12" s="103" t="s">
         <v>414</v>
@@ -2611,15 +2623,15 @@
         <v>413</v>
       </c>
       <c r="G12" s="103" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="103" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="B13" s="103" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="C13" s="103" t="s">
         <v>414</v>
@@ -2631,7 +2643,7 @@
         <v>413</v>
       </c>
       <c r="G13" s="103" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
data(portfolio): onboarding como pre-requisito + pacotes liberam BPL-000
Revisao da Gestora na aba Atributos (pos-B2): BPL-000 vira pre-req de
analise/plano/GDC/mentocoach e os pacotes pleno..embaixador liberam BPL-000.
Primeira mudanca de regra feita puramente por dado — zero codigo; o motor da
Fase B2 aplica. Validado por diff: so preRequisitos/libera mudaram.

Vigora no proximo clique de Sincronizar Portfolio.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portfolio/portfolio_bplen.xlsx
+++ b/portfolio/portfolio_bplen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BPlen_HUB\Dev\portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3B1262-7FC5-4499-B50A-7EF50E1C7BAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5467C438-FCE7-487F-BF5F-135A45D3C8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="728" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="436">
   <si>
     <t>BPlen HUB</t>
   </si>
@@ -1316,34 +1316,40 @@
     <t>Pacote Pleno</t>
   </si>
   <si>
-    <t>BPL-001,BPL-002</t>
-  </si>
-  <si>
     <t>BPL-PAC-SR</t>
   </si>
   <si>
     <t>Pacote Senior</t>
   </si>
   <si>
-    <t>BPL-001,BPL-002,BPL-003</t>
-  </si>
-  <si>
     <t>BPL-PAC-LD</t>
   </si>
   <si>
     <t>Pacote Líder</t>
   </si>
   <si>
-    <t>BPL-001,BPL-002,BPL-003,BPL-004</t>
-  </si>
-  <si>
     <t>BPL-PAC-EB</t>
   </si>
   <si>
     <t>Pacote Embaixador</t>
   </si>
   <si>
-    <t>BPL-001,BPL-002,BPL-003,BPL-004,BPL-005</t>
+    <t>BPL-000,BPL-002</t>
+  </si>
+  <si>
+    <t>BPL-000,BPL-003</t>
+  </si>
+  <si>
+    <t>BPL-000,BPL-001,BPL-002</t>
+  </si>
+  <si>
+    <t>BPL-000,BPL-001,BPL-002,BPL-003</t>
+  </si>
+  <si>
+    <t>BPL-000,BPL-001,BPL-002,BPL-003,BPL-004</t>
+  </si>
+  <si>
+    <t>BPL-000,BPL-001,BPL-002,BPL-003,BPL-004,BPL-005</t>
   </si>
 </sst>
 </file>
@@ -2454,7 +2460,10 @@
         <v>415</v>
       </c>
       <c r="E4" s="103" t="s">
-        <v>413</v>
+        <v>416</v>
+      </c>
+      <c r="F4" s="103" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2474,7 +2483,7 @@
         <v>416</v>
       </c>
       <c r="F5" s="103" t="s">
-        <v>242</v>
+        <v>430</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2494,7 +2503,7 @@
         <v>416</v>
       </c>
       <c r="F6" s="103" t="s">
-        <v>243</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2511,7 +2520,10 @@
         <v>415</v>
       </c>
       <c r="E7" s="103" t="s">
-        <v>413</v>
+        <v>416</v>
+      </c>
+      <c r="F7" s="103" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2571,15 +2583,15 @@
         <v>413</v>
       </c>
       <c r="G10" s="103" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="103" t="s">
+        <v>424</v>
+      </c>
+      <c r="B11" s="103" t="s">
         <v>425</v>
-      </c>
-      <c r="B11" s="103" t="s">
-        <v>426</v>
       </c>
       <c r="C11" s="103" t="s">
         <v>414</v>
@@ -2591,15 +2603,15 @@
         <v>413</v>
       </c>
       <c r="G11" s="103" t="s">
-        <v>427</v>
+        <v>433</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="103" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B12" s="103" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C12" s="103" t="s">
         <v>414</v>
@@ -2611,15 +2623,15 @@
         <v>413</v>
       </c>
       <c r="G12" s="103" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="103" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="B13" s="103" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="C13" s="103" t="s">
         <v>414</v>
@@ -2631,7 +2643,7 @@
         <v>413</v>
       </c>
       <c r="G13" s="103" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>